<commit_message>
Cadrage : graphique EBITDA reel 2024-2026 et budget 2027
Colonnes EBITDA sur quatre exercices, la barre 2027 dans un bleu distinct,
et l'objectif en ligne rouge tiretee comme repere. Le lecteur voit la pente
historique, la marche que produit la construction, et si elle passe au-dessus
de l'objectif.

L'historique est reconstitue depuis l'onglet PNL (comptes 70x moins 6xx hors
6811, soit la definition d'EBITDA deja utilisee par CAD_PIL). Controle : 2026
retombe exactement sur 3 845 790 EUR, et les trois versions 2027 sur
4 111 492 / 6 744 292 / 2 329 565 EUR.

La zone de donnees du graphique est en P4:S9, hors zone d'impression.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/CAD_PIL_MEP.xlsx
+++ b/eduservices/CAD_PIL_MEP.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Cadrage'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cadrage'!$A$1:$F$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cadrage'!$A$1:$M$44</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Pilotage'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Pilotage'!$A$1:$L$57</definedName>
   </definedNames>
@@ -29,7 +29,7 @@
     <numFmt numFmtId="167" formatCode="0.00%;[Red]-0.00%"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,6 +103,12 @@
       <name val="Arial"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -305,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -315,6 +321,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -326,6 +335,15 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -444,7 +462,7 @@
     <xf numFmtId="2" fontId="3" fillId="3" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -454,42 +472,42 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="15" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="15" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -566,6 +584,224 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>EBITDA : réel 2024-2026 et budget 2027</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cadrage'!Q5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3B57"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cadrage'!$P$6:$P$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cadrage'!$Q$6:$Q$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Cadrage'!R5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cadrage'!$P$6:$P$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cadrage'!$R$6:$R$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="#,##0"/>
+          <txPr>
+            <a:bodyPr/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="800">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Cadrage'!S5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="18000">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Cadrage'!$S$6:$S$9</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0&quot; €&quot;" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3744000" cy="2556000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -873,6 +1109,10 @@
     <col width="9.5" customWidth="1" min="11" max="11"/>
     <col width="2" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1">
@@ -962,30 +1202,34 @@
       <c r="M4" s="1" t="n"/>
       <c r="N4" s="1" t="n"/>
       <c r="O4" s="1" t="n"/>
-      <c r="P4" s="1" t="n"/>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>Données du graphique</t>
+        </is>
+      </c>
       <c r="Q4" s="1" t="n"/>
       <c r="R4" s="1" t="n"/>
       <c r="S4" s="1" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Scénario retenu</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Optimiste</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Objectif de croissance EBITDA</t>
         </is>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="9" t="n">
         <v>0.065</v>
       </c>
       <c r="G5" s="1" t="n"/>
@@ -997,10 +1241,26 @@
       <c r="M5" s="1" t="n"/>
       <c r="N5" s="1" t="n"/>
       <c r="O5" s="1" t="n"/>
-      <c r="P5" s="1" t="n"/>
-      <c r="Q5" s="1" t="n"/>
-      <c r="R5" s="1" t="n"/>
-      <c r="S5" s="1" t="n"/>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Exercice</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>Réel</t>
+        </is>
+      </c>
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>Budget 2027</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>Objectif</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="12" customHeight="1">
       <c r="A6" s="1" t="n"/>
@@ -1018,30 +1278,36 @@
       <c r="M6" s="1" t="n"/>
       <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="n"/>
-      <c r="P6" s="1" t="n"/>
-      <c r="Q6" s="1" t="n"/>
+      <c r="P6" s="11" t="n">
+        <v>2024</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>3151035</v>
+      </c>
       <c r="R6" s="1" t="n"/>
-      <c r="S6" s="1" t="n"/>
+      <c r="S6" s="12" t="n">
+        <v>4095766.36</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="n"/>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Objectif EBITDA 2027</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>EBITDA construit</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Écart à l'objectif</t>
         </is>
       </c>
-      <c r="F7" s="12" t="n"/>
+      <c r="F7" s="16" t="n"/>
       <c r="G7" s="1" t="n"/>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
@@ -1051,24 +1317,30 @@
       <c r="M7" s="1" t="n"/>
       <c r="N7" s="1" t="n"/>
       <c r="O7" s="1" t="n"/>
-      <c r="P7" s="1" t="n"/>
-      <c r="Q7" s="1" t="n"/>
+      <c r="P7" s="11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>3467768</v>
+      </c>
       <c r="R7" s="1" t="n"/>
-      <c r="S7" s="1" t="n"/>
+      <c r="S7" s="12" t="n">
+        <v>4095766.36</v>
+      </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="17" t="n">
         <v>4095766.36</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="18" t="n">
         <v>6744302.91</v>
       </c>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="14" t="n">
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="18" t="n">
         <v>2648536.55</v>
       </c>
-      <c r="F8" s="16" t="n"/>
+      <c r="F8" s="20" t="n"/>
       <c r="G8" s="1" t="n"/>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
@@ -1078,30 +1350,36 @@
       <c r="M8" s="1" t="n"/>
       <c r="N8" s="1" t="n"/>
       <c r="O8" s="1" t="n"/>
-      <c r="P8" s="1" t="n"/>
-      <c r="Q8" s="1" t="n"/>
+      <c r="P8" s="11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="Q8" s="12" t="n">
+        <v>3845790</v>
+      </c>
       <c r="R8" s="1" t="n"/>
-      <c r="S8" s="1" t="n"/>
+      <c r="S8" s="12" t="n">
+        <v>4095766.36</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>2026 : 3 845 790 €</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>marge 25,2 %</t>
         </is>
       </c>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="D9" s="23" t="n"/>
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>objectif dépassé</t>
         </is>
       </c>
-      <c r="F9" s="20" t="n"/>
+      <c r="F9" s="24" t="n"/>
       <c r="G9" s="1" t="n"/>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
@@ -1111,22 +1389,28 @@
       <c r="M9" s="1" t="n"/>
       <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="n"/>
-      <c r="P9" s="1" t="n"/>
+      <c r="P9" s="11" t="n">
+        <v>2027</v>
+      </c>
       <c r="Q9" s="1" t="n"/>
-      <c r="R9" s="1" t="n"/>
-      <c r="S9" s="1" t="n"/>
+      <c r="R9" s="12" t="n">
+        <v>6744302.91</v>
+      </c>
+      <c r="S9" s="12" t="n">
+        <v>4095766.36</v>
+      </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>RÉCONCILIATION 2026 / 2027</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="22" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="26" t="n"/>
       <c r="G10" s="1" t="n"/>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
@@ -1143,27 +1427,27 @@
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="28" t="inlineStr">
         <is>
           <t>Réel 2026</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="28" t="inlineStr">
         <is>
           <t>Budget 2027</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>Écart</t>
         </is>
       </c>
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F11" s="28" t="inlineStr">
         <is>
           <t>Écart %</t>
         </is>
@@ -1184,21 +1468,21 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="30" t="n">
         <v>23098985</v>
       </c>
-      <c r="D12" s="26" t="n">
+      <c r="D12" s="30" t="n">
         <v>26814168.68</v>
       </c>
-      <c r="E12" s="26" t="n">
+      <c r="E12" s="30" t="n">
         <v>3715183.68</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="31" t="n">
         <v>0.1608</v>
       </c>
       <c r="G12" s="1" t="n"/>
@@ -1217,21 +1501,21 @@
     </row>
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C13" s="29" t="n">
+      <c r="C13" s="33" t="n">
         <v>3845790.01</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="33" t="n">
         <v>6744302.91</v>
       </c>
-      <c r="E13" s="29" t="n">
+      <c r="E13" s="33" t="n">
         <v>2898512.9</v>
       </c>
-      <c r="F13" s="30" t="n">
+      <c r="F13" s="34" t="n">
         <v>0.7537</v>
       </c>
       <c r="G13" s="1" t="n"/>
@@ -1250,21 +1534,21 @@
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>Marge EBITDA</t>
         </is>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="31" t="n">
         <v>0.1665</v>
       </c>
-      <c r="D14" s="27" t="n">
+      <c r="D14" s="31" t="n">
         <v>0.2515</v>
       </c>
-      <c r="E14" s="27" t="n">
+      <c r="E14" s="31" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="F14" s="31" t="n"/>
+      <c r="F14" s="35" t="n"/>
       <c r="G14" s="1" t="n"/>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
@@ -1281,21 +1565,21 @@
     </row>
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="25" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>Effectif moyen</t>
         </is>
       </c>
-      <c r="C15" s="32" t="n">
+      <c r="C15" s="36" t="n">
         <v>3114</v>
       </c>
-      <c r="D15" s="32" t="n">
+      <c r="D15" s="36" t="n">
         <v>3473.67</v>
       </c>
-      <c r="E15" s="32" t="n">
+      <c r="E15" s="36" t="n">
         <v>359.67</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="31" t="n">
         <v>0.1155</v>
       </c>
       <c r="G15" s="1" t="n"/>
@@ -1356,15 +1640,15 @@
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>HYPOTHÈSES DE CONSTRUCTION</t>
         </is>
       </c>
-      <c r="C18" s="22" t="n"/>
-      <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="22" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="26" t="n"/>
       <c r="G18" s="1" t="n"/>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="1" t="n"/>
@@ -1381,27 +1665,27 @@
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="1" t="n"/>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>Levier</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C19" s="37" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="D19" s="33" t="inlineStr">
+      <c r="D19" s="37" t="inlineStr">
         <is>
           <t>Optimiste</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr">
+      <c r="E19" s="37" t="inlineStr">
         <is>
           <t>Prudent</t>
         </is>
       </c>
-      <c r="F19" s="34" t="inlineStr">
+      <c r="F19" s="38" t="inlineStr">
         <is>
           <t>Retenu</t>
         </is>
@@ -1443,24 +1727,24 @@
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="1" t="n"/>
-      <c r="B21" s="35" t="inlineStr">
+      <c r="B21" s="39" t="inlineStr">
         <is>
           <t>Croissance</t>
         </is>
       </c>
-      <c r="C21" s="36" t="n"/>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="36" t="n"/>
-      <c r="F21" s="36" t="n"/>
+      <c r="C21" s="40" t="n"/>
+      <c r="D21" s="40" t="n"/>
+      <c r="E21" s="40" t="n"/>
+      <c r="F21" s="40" t="n"/>
       <c r="G21" s="1" t="n"/>
       <c r="H21" s="1" t="n"/>
       <c r="I21" s="1" t="n"/>
-      <c r="J21" s="21" t="inlineStr">
+      <c r="J21" s="25" t="inlineStr">
         <is>
           <t>COEFFICIENTS DE PRIX</t>
         </is>
       </c>
-      <c r="K21" s="22" t="n"/>
+      <c r="K21" s="26" t="n"/>
       <c r="L21" s="1" t="n"/>
       <c r="M21" s="1" t="n"/>
       <c r="N21" s="1" t="n"/>
@@ -1473,17 +1757,17 @@
     <row r="22" ht="9" customHeight="1">
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="1" t="n"/>
-      <c r="C22" s="37" t="inlineStr">
+      <c r="C22" s="41" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="D22" s="37" t="inlineStr">
+      <c r="D22" s="41" t="inlineStr">
         <is>
           <t>Optimiste</t>
         </is>
       </c>
-      <c r="E22" s="37" t="inlineStr">
+      <c r="E22" s="41" t="inlineStr">
         <is>
           <t>Prudent</t>
         </is>
@@ -1505,32 +1789,32 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="25" t="inlineStr">
+      <c r="B23" s="29" t="inlineStr">
         <is>
           <t>Variation du budget d'acquisition</t>
         </is>
       </c>
-      <c r="C23" s="38" t="n">
+      <c r="C23" s="42" t="n">
         <v>0.08</v>
       </c>
-      <c r="D23" s="38" t="n">
+      <c r="D23" s="42" t="n">
         <v>0.15</v>
       </c>
-      <c r="E23" s="38" t="n">
+      <c r="E23" s="42" t="n">
         <v>-0.05</v>
       </c>
-      <c r="F23" s="39" t="n">
+      <c r="F23" s="43" t="n">
         <v>0.15</v>
       </c>
       <c r="G23" s="1" t="n"/>
       <c r="H23" s="1" t="n"/>
       <c r="I23" s="1" t="n"/>
-      <c r="J23" s="23" t="inlineStr">
+      <c r="J23" s="27" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="K23" s="33" t="inlineStr">
+      <c r="K23" s="37" t="inlineStr">
         <is>
           <t>Coeff.</t>
         </is>
@@ -1546,32 +1830,32 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="B24" s="29" t="inlineStr">
         <is>
           <t>Variation du budget de marque</t>
         </is>
       </c>
-      <c r="C24" s="38" t="n">
+      <c r="C24" s="42" t="n">
         <v>0.1</v>
       </c>
-      <c r="D24" s="38" t="n">
+      <c r="D24" s="42" t="n">
         <v>0.15</v>
       </c>
-      <c r="E24" s="38" t="n">
+      <c r="E24" s="42" t="n">
         <v>-0.05</v>
       </c>
-      <c r="F24" s="39" t="n">
+      <c r="F24" s="43" t="n">
         <v>0.15</v>
       </c>
       <c r="G24" s="1" t="n"/>
       <c r="H24" s="1" t="n"/>
       <c r="I24" s="1" t="n"/>
-      <c r="J24" s="25" t="inlineStr">
+      <c r="J24" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="K24" s="40" t="n">
+      <c r="K24" s="44" t="n">
         <v>1.2</v>
       </c>
       <c r="L24" s="1" t="n"/>
@@ -1585,32 +1869,32 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>Hausse tarifaire</t>
         </is>
       </c>
-      <c r="C25" s="38" t="n">
+      <c r="C25" s="42" t="n">
         <v>0.0029</v>
       </c>
-      <c r="D25" s="38" t="n">
+      <c r="D25" s="42" t="n">
         <v>0.035</v>
       </c>
-      <c r="E25" s="38" t="n">
+      <c r="E25" s="42" t="n">
         <v>0.02</v>
       </c>
-      <c r="F25" s="39" t="n">
+      <c r="F25" s="43" t="n">
         <v>0.035</v>
       </c>
       <c r="G25" s="1" t="n"/>
       <c r="H25" s="1" t="n"/>
       <c r="I25" s="1" t="n"/>
-      <c r="J25" s="25" t="inlineStr">
+      <c r="J25" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="K25" s="40" t="n">
+      <c r="K25" s="44" t="n">
         <v>1.15</v>
       </c>
       <c r="L25" s="1" t="n"/>
@@ -1624,32 +1908,32 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="25" t="inlineStr">
+      <c r="B26" s="29" t="inlineStr">
         <is>
           <t>Gain de conversion lead / candidature</t>
         </is>
       </c>
-      <c r="C26" s="38" t="n">
+      <c r="C26" s="42" t="n">
         <v>0.01</v>
       </c>
-      <c r="D26" s="38" t="n">
+      <c r="D26" s="42" t="n">
         <v>0.03</v>
       </c>
-      <c r="E26" s="38" t="n">
+      <c r="E26" s="42" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F26" s="39" t="n">
+      <c r="F26" s="43" t="n">
         <v>0.03</v>
       </c>
       <c r="G26" s="1" t="n"/>
       <c r="H26" s="1" t="n"/>
       <c r="I26" s="1" t="n"/>
-      <c r="J26" s="25" t="inlineStr">
+      <c r="J26" s="29" t="inlineStr">
         <is>
           <t>Ipac Bachelor Factory</t>
         </is>
       </c>
-      <c r="K26" s="40" t="n">
+      <c r="K26" s="44" t="n">
         <v>0.95</v>
       </c>
       <c r="L26" s="1" t="n"/>
@@ -1663,32 +1947,32 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="25" t="inlineStr">
+      <c r="B27" s="29" t="inlineStr">
         <is>
           <t>Gain de conversion admis / inscrit</t>
         </is>
       </c>
-      <c r="C27" s="38" t="n">
+      <c r="C27" s="42" t="n">
         <v>0.01</v>
       </c>
-      <c r="D27" s="38" t="n">
+      <c r="D27" s="42" t="n">
         <v>0.025</v>
       </c>
-      <c r="E27" s="38" t="n">
+      <c r="E27" s="42" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F27" s="39" t="n">
+      <c r="F27" s="43" t="n">
         <v>0.025</v>
       </c>
       <c r="G27" s="1" t="n"/>
       <c r="H27" s="1" t="n"/>
       <c r="I27" s="1" t="n"/>
-      <c r="J27" s="25" t="inlineStr">
+      <c r="J27" s="29" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="K27" s="40" t="n">
+      <c r="K27" s="44" t="n">
         <v>0.9</v>
       </c>
       <c r="L27" s="1" t="n"/>
@@ -1702,32 +1986,32 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="25" t="inlineStr">
+      <c r="B28" s="29" t="inlineStr">
         <is>
           <t>Amélioration du taux de passage</t>
         </is>
       </c>
-      <c r="C28" s="38" t="n">
+      <c r="C28" s="42" t="n">
         <v>0.005</v>
       </c>
-      <c r="D28" s="38" t="n">
+      <c r="D28" s="42" t="n">
         <v>0.015</v>
       </c>
-      <c r="E28" s="38" t="n">
+      <c r="E28" s="42" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F28" s="39" t="n">
+      <c r="F28" s="43" t="n">
         <v>0.015</v>
       </c>
       <c r="G28" s="1" t="n"/>
       <c r="H28" s="1" t="n"/>
       <c r="I28" s="1" t="n"/>
-      <c r="J28" s="25" t="inlineStr">
+      <c r="J28" s="29" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="K28" s="40" t="n">
+      <c r="K28" s="44" t="n">
         <v>1.05</v>
       </c>
       <c r="L28" s="1" t="n"/>
@@ -1804,15 +2088,15 @@
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="35" t="inlineStr">
+      <c r="B32" s="39" t="inlineStr">
         <is>
           <t>Coûts</t>
         </is>
       </c>
-      <c r="C32" s="36" t="n"/>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="36" t="n"/>
-      <c r="F32" s="36" t="n"/>
+      <c r="C32" s="40" t="n"/>
+      <c r="D32" s="40" t="n"/>
+      <c r="E32" s="40" t="n"/>
+      <c r="F32" s="40" t="n"/>
       <c r="G32" s="1" t="n"/>
       <c r="H32" s="1" t="n"/>
       <c r="I32" s="1" t="n"/>
@@ -1850,21 +2134,21 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="n"/>
-      <c r="B34" s="25" t="inlineStr">
+      <c r="B34" s="29" t="inlineStr">
         <is>
           <t>Inflation des charges externes</t>
         </is>
       </c>
-      <c r="C34" s="38" t="n">
+      <c r="C34" s="42" t="n">
         <v>0.02</v>
       </c>
-      <c r="D34" s="38" t="n">
+      <c r="D34" s="42" t="n">
         <v>0.015</v>
       </c>
-      <c r="E34" s="38" t="n">
+      <c r="E34" s="42" t="n">
         <v>0.03</v>
       </c>
-      <c r="F34" s="39" t="n">
+      <c r="F34" s="43" t="n">
         <v>0.015</v>
       </c>
       <c r="G34" s="1" t="n"/>
@@ -1883,21 +2167,21 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="25" t="inlineStr">
+      <c r="B35" s="29" t="inlineStr">
         <is>
           <t>Politique salariale</t>
         </is>
       </c>
-      <c r="C35" s="38" t="n">
+      <c r="C35" s="42" t="n">
         <v>0.025</v>
       </c>
-      <c r="D35" s="38" t="n">
+      <c r="D35" s="42" t="n">
         <v>0.02</v>
       </c>
-      <c r="E35" s="38" t="n">
+      <c r="E35" s="42" t="n">
         <v>0.03</v>
       </c>
-      <c r="F35" s="39" t="n">
+      <c r="F35" s="43" t="n">
         <v>0.02</v>
       </c>
       <c r="G35" s="1" t="n"/>
@@ -1916,21 +2200,21 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="B36" s="29" t="inlineStr">
         <is>
           <t>Variation des effectifs permanents</t>
         </is>
       </c>
-      <c r="C36" s="38" t="n">
+      <c r="C36" s="42" t="n">
         <v>0.04</v>
       </c>
-      <c r="D36" s="38" t="n">
+      <c r="D36" s="42" t="n">
         <v>0.03</v>
       </c>
-      <c r="E36" s="38" t="n">
+      <c r="E36" s="42" t="n">
         <v>0.05</v>
       </c>
-      <c r="F36" s="39" t="n">
+      <c r="F36" s="43" t="n">
         <v>0.03</v>
       </c>
       <c r="G36" s="1" t="n"/>
@@ -1949,23 +2233,23 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="25" t="inlineStr">
+      <c r="B37" s="29" t="inlineStr">
         <is>
           <t>Effort de productivité</t>
         </is>
       </c>
-      <c r="C37" s="38" t="n">
+      <c r="C37" s="42" t="n">
         <v>0.0185</v>
       </c>
-      <c r="D37" s="38" t="n">
+      <c r="D37" s="42" t="n">
         <v>0.03</v>
       </c>
-      <c r="E37" s="41" t="inlineStr">
+      <c r="E37" s="45" t="inlineStr">
         <is>
           <t>n.d.</t>
         </is>
       </c>
-      <c r="F37" s="39" t="n">
+      <c r="F37" s="43" t="n">
         <v>0.03</v>
       </c>
       <c r="G37" s="1" t="n"/>
@@ -1984,23 +2268,23 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="25" t="inlineStr">
+      <c r="B38" s="29" t="inlineStr">
         <is>
           <t>Variation des coûts de structure</t>
         </is>
       </c>
-      <c r="C38" s="41" t="inlineStr">
+      <c r="C38" s="45" t="inlineStr">
         <is>
           <t>n.d.</t>
         </is>
       </c>
-      <c r="D38" s="38" t="n">
+      <c r="D38" s="42" t="n">
         <v>-0.03</v>
       </c>
-      <c r="E38" s="38" t="n">
+      <c r="E38" s="42" t="n">
         <v>0.04</v>
       </c>
-      <c r="F38" s="39" t="n">
+      <c r="F38" s="43" t="n">
         <v>-0.03</v>
       </c>
       <c r="G38" s="1" t="n"/>
@@ -2040,15 +2324,15 @@
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="35" t="inlineStr">
+      <c r="B40" s="39" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="C40" s="36" t="n"/>
-      <c r="D40" s="36" t="n"/>
-      <c r="E40" s="36" t="n"/>
-      <c r="F40" s="36" t="n"/>
+      <c r="C40" s="40" t="n"/>
+      <c r="D40" s="40" t="n"/>
+      <c r="E40" s="40" t="n"/>
+      <c r="F40" s="40" t="n"/>
       <c r="G40" s="1" t="n"/>
       <c r="H40" s="1" t="n"/>
       <c r="I40" s="1" t="n"/>
@@ -2086,21 +2370,21 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="n"/>
-      <c r="B42" s="25" t="inlineStr">
+      <c r="B42" s="29" t="inlineStr">
         <is>
           <t>Frais de dossier par nouvel inscrit</t>
         </is>
       </c>
-      <c r="C42" s="42" t="n">
+      <c r="C42" s="46" t="n">
         <v>90</v>
       </c>
-      <c r="D42" s="42" t="n">
+      <c r="D42" s="46" t="n">
         <v>90</v>
       </c>
-      <c r="E42" s="42" t="n">
+      <c r="E42" s="46" t="n">
         <v>90</v>
       </c>
-      <c r="F42" s="43" t="n">
+      <c r="F42" s="47" t="n">
         <v>90</v>
       </c>
       <c r="G42" s="1" t="n"/>
@@ -2140,7 +2424,7 @@
     </row>
     <row r="44" ht="12" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="44" t="inlineStr">
+      <c r="B44" s="48" t="inlineStr">
         <is>
           <t>Source : Tagetik TGK_MSSQL_07, cube d'hypothèses, versions V01 / V02 / V03.</t>
         </is>
@@ -2213,6 +2497,7 @@
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2379,14 +2664,14 @@
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Scénario retenu</t>
         </is>
       </c>
       <c r="C6" s="1" t="n"/>
       <c r="D6" s="1" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
@@ -2462,36 +2747,36 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>EBITDA après siège</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Marge EBITDA</t>
         </is>
       </c>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Effectif moyen</t>
         </is>
       </c>
-      <c r="H9" s="11" t="n"/>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>Croissance CA</t>
         </is>
       </c>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="12" t="n"/>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="16" t="n"/>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
       <c r="N9" s="1" t="n"/>
@@ -2507,26 +2792,26 @@
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="17" t="n">
         <v>24231703.55</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="18" t="n">
         <v>4111503.64</v>
       </c>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="45" t="n">
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="49" t="n">
         <v>0.1697</v>
       </c>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="46" t="n">
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="50" t="n">
         <v>3253.62</v>
       </c>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="45" t="n">
+      <c r="H10" s="19" t="n"/>
+      <c r="I10" s="49" t="n">
         <v>0.049</v>
       </c>
-      <c r="J10" s="15" t="n"/>
-      <c r="K10" s="16" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="20" t="n"/>
       <c r="L10" s="1" t="n"/>
       <c r="M10" s="1" t="n"/>
       <c r="N10" s="1" t="n"/>
@@ -2542,36 +2827,36 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>2026 : 23 098 985 €</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>2026 : 3 845 790 €</t>
         </is>
       </c>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="D11" s="23" t="n"/>
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>2026 : 16,6 %</t>
         </is>
       </c>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>2026 : 3 114</t>
         </is>
       </c>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="18" t="inlineStr">
+      <c r="H11" s="23" t="n"/>
+      <c r="I11" s="22" t="inlineStr">
         <is>
           <t>vs réel 2026</t>
         </is>
       </c>
-      <c r="J11" s="19" t="n"/>
-      <c r="K11" s="20" t="n"/>
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="24" t="n"/>
       <c r="L11" s="1" t="n"/>
       <c r="M11" s="1" t="n"/>
       <c r="N11" s="1" t="n"/>
@@ -2687,21 +2972,21 @@
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>CAPACITÉ PAR CAMPUS</t>
         </is>
       </c>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="22" t="n"/>
-      <c r="G16" s="22" t="n"/>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="22" t="n"/>
-      <c r="J16" s="22" t="n"/>
-      <c r="K16" s="22" t="n"/>
-      <c r="L16" s="22" t="n"/>
+      <c r="C16" s="26" t="n"/>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="26" t="n"/>
+      <c r="F16" s="26" t="n"/>
+      <c r="G16" s="26" t="n"/>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="26" t="n"/>
+      <c r="J16" s="26" t="n"/>
+      <c r="K16" s="26" t="n"/>
+      <c r="L16" s="26" t="n"/>
       <c r="M16" s="1" t="n"/>
       <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
@@ -2740,58 +3025,58 @@
       <c r="W17" s="1" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="47" t="inlineStr"/>
-      <c r="B18" s="48" t="inlineStr">
+      <c r="A18" s="51" t="inlineStr"/>
+      <c r="B18" s="52" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="C18" s="48" t="inlineStr">
+      <c r="C18" s="52" t="inlineStr">
         <is>
           <t>Ville</t>
         </is>
       </c>
-      <c r="D18" s="49" t="inlineStr">
+      <c r="D18" s="53" t="inlineStr">
         <is>
           <t>CAC marginal</t>
         </is>
       </c>
-      <c r="E18" s="49" t="inlineStr">
+      <c r="E18" s="53" t="inlineStr">
         <is>
           <t>Croissance leads</t>
         </is>
       </c>
-      <c r="F18" s="49" t="inlineStr">
+      <c r="F18" s="53" t="inlineStr">
         <is>
           <t>Intensité marketing</t>
         </is>
       </c>
-      <c r="G18" s="47" t="inlineStr">
+      <c r="G18" s="51" t="inlineStr">
         <is>
           <t>Cap effectif</t>
         </is>
       </c>
-      <c r="H18" s="47" t="inlineStr">
+      <c r="H18" s="51" t="inlineStr">
         <is>
           <t>Cap momentum</t>
         </is>
       </c>
-      <c r="I18" s="47" t="inlineStr">
+      <c r="I18" s="51" t="inlineStr">
         <is>
           <t>Cap potentiel</t>
         </is>
       </c>
-      <c r="J18" s="50" t="inlineStr">
+      <c r="J18" s="54" t="inlineStr">
         <is>
           <t>Cap retenu</t>
         </is>
       </c>
-      <c r="K18" s="49" t="inlineStr">
+      <c r="K18" s="53" t="inlineStr">
         <is>
           <t>Budget acquisition</t>
         </is>
       </c>
-      <c r="L18" s="48" t="inlineStr">
+      <c r="L18" s="52" t="inlineStr">
         <is>
           <t>Code campus</t>
         </is>
@@ -2809,42 +3094,42 @@
       <c r="W18" s="1" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="51" t="inlineStr"/>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="A19" s="55" t="inlineStr"/>
+      <c r="B19" s="29" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C19" s="52" t="inlineStr">
+      <c r="C19" s="56" t="inlineStr">
         <is>
           <t>Montpellier</t>
         </is>
       </c>
-      <c r="D19" s="26" t="n">
+      <c r="D19" s="30" t="n">
         <v>1033.98</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E19" s="31" t="n">
         <v>0.1448</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="31" t="n">
         <v>0.0194</v>
       </c>
-      <c r="G19" s="40" t="n">
+      <c r="G19" s="44" t="n">
         <v>1.1626</v>
       </c>
-      <c r="H19" s="40" t="n">
+      <c r="H19" s="44" t="n">
         <v>1.3855</v>
       </c>
-      <c r="I19" s="40" t="n">
+      <c r="I19" s="44" t="n">
         <v>0.9443</v>
       </c>
-      <c r="J19" s="53" t="n">
+      <c r="J19" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K19" s="26" t="n">
+      <c r="K19" s="30" t="n">
         <v>15178</v>
       </c>
-      <c r="L19" s="54" t="inlineStr">
+      <c r="L19" s="58" t="inlineStr">
         <is>
           <t>IPAC_MTP</t>
         </is>
@@ -2862,42 +3147,42 @@
       <c r="W19" s="1" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="51" t="inlineStr"/>
-      <c r="B20" s="25" t="inlineStr">
+      <c r="A20" s="55" t="inlineStr"/>
+      <c r="B20" s="29" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C20" s="52" t="inlineStr">
+      <c r="C20" s="56" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D20" s="26" t="n">
+      <c r="D20" s="30" t="n">
         <v>1216.29</v>
       </c>
-      <c r="E20" s="27" t="n">
+      <c r="E20" s="31" t="n">
         <v>0.1379</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="31" t="n">
         <v>0.0213</v>
       </c>
-      <c r="G20" s="40" t="n">
+      <c r="G20" s="44" t="n">
         <v>0.9883</v>
       </c>
-      <c r="H20" s="40" t="n">
+      <c r="H20" s="44" t="n">
         <v>1.3195</v>
       </c>
-      <c r="I20" s="40" t="n">
+      <c r="I20" s="44" t="n">
         <v>0.8591</v>
       </c>
-      <c r="J20" s="53" t="n">
+      <c r="J20" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K20" s="26" t="n">
+      <c r="K20" s="30" t="n">
         <v>21760</v>
       </c>
-      <c r="L20" s="54" t="inlineStr">
+      <c r="L20" s="58" t="inlineStr">
         <is>
           <t>IPAC_NAN</t>
         </is>
@@ -2915,42 +3200,42 @@
       <c r="W20" s="1" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="51" t="inlineStr"/>
-      <c r="B21" s="25" t="inlineStr">
+      <c r="A21" s="55" t="inlineStr"/>
+      <c r="B21" s="29" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C21" s="52" t="inlineStr">
+      <c r="C21" s="56" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="D21" s="26" t="n">
+      <c r="D21" s="30" t="n">
         <v>1040.56</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E21" s="31" t="n">
         <v>0.1448</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F21" s="31" t="n">
         <v>0.0191</v>
       </c>
-      <c r="G21" s="40" t="n">
+      <c r="G21" s="44" t="n">
         <v>1.1553</v>
       </c>
-      <c r="H21" s="40" t="n">
+      <c r="H21" s="44" t="n">
         <v>1.3855</v>
       </c>
-      <c r="I21" s="40" t="n">
+      <c r="I21" s="44" t="n">
         <v>0.9598</v>
       </c>
-      <c r="J21" s="53" t="n">
+      <c r="J21" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K21" s="26" t="n">
+      <c r="K21" s="30" t="n">
         <v>14933</v>
       </c>
-      <c r="L21" s="54" t="inlineStr">
+      <c r="L21" s="58" t="inlineStr">
         <is>
           <t>IPAC_REN</t>
         </is>
@@ -2968,42 +3253,42 @@
       <c r="W21" s="1" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="51" t="inlineStr"/>
-      <c r="B22" s="25" t="inlineStr">
+      <c r="A22" s="55" t="inlineStr"/>
+      <c r="B22" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C22" s="52" t="inlineStr">
+      <c r="C22" s="56" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="D22" s="26" t="n">
+      <c r="D22" s="30" t="n">
         <v>978.58</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="31" t="n">
         <v>0.0815</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="31" t="n">
         <v>0.0144</v>
       </c>
-      <c r="G22" s="40" t="n">
+      <c r="G22" s="44" t="n">
         <v>1.2284</v>
       </c>
-      <c r="H22" s="40" t="n">
+      <c r="H22" s="44" t="n">
         <v>0.7804</v>
       </c>
-      <c r="I22" s="40" t="n">
+      <c r="I22" s="44" t="n">
         <v>1.2767</v>
       </c>
-      <c r="J22" s="53" t="n">
+      <c r="J22" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="26" t="n">
+      <c r="K22" s="30" t="n">
         <v>25220</v>
       </c>
-      <c r="L22" s="54" t="inlineStr">
+      <c r="L22" s="58" t="inlineStr">
         <is>
           <t>ISCOM_LIL</t>
         </is>
@@ -3021,42 +3306,42 @@
       <c r="W22" s="1" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="51" t="inlineStr"/>
-      <c r="B23" s="25" t="inlineStr">
+      <c r="A23" s="55" t="inlineStr"/>
+      <c r="B23" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C23" s="52" t="inlineStr">
+      <c r="C23" s="56" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D23" s="26" t="n">
+      <c r="D23" s="30" t="n">
         <v>1540.33</v>
       </c>
-      <c r="E23" s="27" t="n">
+      <c r="E23" s="31" t="n">
         <v>0.07770000000000001</v>
       </c>
-      <c r="F23" s="27" t="n">
+      <c r="F23" s="31" t="n">
         <v>0.0209</v>
       </c>
-      <c r="G23" s="40" t="n">
+      <c r="G23" s="44" t="n">
         <v>0.7804</v>
       </c>
-      <c r="H23" s="40" t="n">
+      <c r="H23" s="44" t="n">
         <v>0.744</v>
       </c>
-      <c r="I23" s="40" t="n">
+      <c r="I23" s="44" t="n">
         <v>0.8773</v>
       </c>
-      <c r="J23" s="53" t="n">
+      <c r="J23" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K23" s="26" t="n">
+      <c r="K23" s="30" t="n">
         <v>60800</v>
       </c>
-      <c r="L23" s="54" t="inlineStr">
+      <c r="L23" s="58" t="inlineStr">
         <is>
           <t>ISCOM_PAR</t>
         </is>
@@ -3074,42 +3359,42 @@
       <c r="W23" s="1" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="51" t="inlineStr"/>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="A24" s="55" t="inlineStr"/>
+      <c r="B24" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C24" s="52" t="inlineStr">
+      <c r="C24" s="56" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="D24" s="26" t="n">
+      <c r="D24" s="30" t="n">
         <v>919.03</v>
       </c>
-      <c r="E24" s="27" t="n">
+      <c r="E24" s="31" t="n">
         <v>0.08210000000000001</v>
       </c>
-      <c r="F24" s="27" t="n">
+      <c r="F24" s="31" t="n">
         <v>0.0136</v>
       </c>
-      <c r="G24" s="40" t="n">
+      <c r="G24" s="44" t="n">
         <v>1.308</v>
       </c>
-      <c r="H24" s="40" t="n">
+      <c r="H24" s="44" t="n">
         <v>0.7858000000000001</v>
       </c>
-      <c r="I24" s="40" t="n">
+      <c r="I24" s="44" t="n">
         <v>1.3518</v>
       </c>
-      <c r="J24" s="53" t="n">
+      <c r="J24" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K24" s="26" t="n">
+      <c r="K24" s="30" t="n">
         <v>22083</v>
       </c>
-      <c r="L24" s="54" t="inlineStr">
+      <c r="L24" s="58" t="inlineStr">
         <is>
           <t>ISCOM_TLS</t>
         </is>
@@ -3127,42 +3412,42 @@
       <c r="W24" s="1" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="51" t="inlineStr"/>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="A25" s="55" t="inlineStr"/>
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C25" s="52" t="inlineStr">
+      <c r="C25" s="56" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D25" s="26" t="n">
+      <c r="D25" s="30" t="n">
         <v>889.59</v>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E25" s="31" t="n">
         <v>0.1261</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="31" t="n">
         <v>0.0141</v>
       </c>
-      <c r="G25" s="40" t="n">
+      <c r="G25" s="44" t="n">
         <v>1.3513</v>
       </c>
-      <c r="H25" s="40" t="n">
+      <c r="H25" s="44" t="n">
         <v>1.2067</v>
       </c>
-      <c r="I25" s="40" t="n">
+      <c r="I25" s="44" t="n">
         <v>1.3049</v>
       </c>
-      <c r="J25" s="53" t="n">
+      <c r="J25" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="26" t="n">
+      <c r="K25" s="30" t="n">
         <v>24923</v>
       </c>
-      <c r="L25" s="54" t="inlineStr">
+      <c r="L25" s="58" t="inlineStr">
         <is>
           <t>MBWAY_BOR</t>
         </is>
@@ -3180,42 +3465,42 @@
       <c r="W25" s="1" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="51" t="inlineStr"/>
-      <c r="B26" s="25" t="inlineStr">
+      <c r="A26" s="55" t="inlineStr"/>
+      <c r="B26" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C26" s="52" t="inlineStr">
+      <c r="C26" s="56" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D26" s="26" t="n">
+      <c r="D26" s="30" t="n">
         <v>1101.6</v>
       </c>
-      <c r="E26" s="27" t="n">
+      <c r="E26" s="31" t="n">
         <v>0.1189</v>
       </c>
-      <c r="F26" s="27" t="n">
+      <c r="F26" s="31" t="n">
         <v>0.0167</v>
       </c>
-      <c r="G26" s="40" t="n">
+      <c r="G26" s="44" t="n">
         <v>1.0912</v>
       </c>
-      <c r="H26" s="40" t="n">
+      <c r="H26" s="44" t="n">
         <v>1.1376</v>
       </c>
-      <c r="I26" s="40" t="n">
+      <c r="I26" s="44" t="n">
         <v>1.0957</v>
       </c>
-      <c r="J26" s="53" t="n">
+      <c r="J26" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K26" s="26" t="n">
+      <c r="K26" s="30" t="n">
         <v>41783</v>
       </c>
-      <c r="L26" s="54" t="inlineStr">
+      <c r="L26" s="58" t="inlineStr">
         <is>
           <t>MBWAY_LYO</t>
         </is>
@@ -3233,42 +3518,42 @@
       <c r="W26" s="1" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="51" t="inlineStr"/>
-      <c r="B27" s="25" t="inlineStr">
+      <c r="A27" s="55" t="inlineStr"/>
+      <c r="B27" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C27" s="52" t="inlineStr">
+      <c r="C27" s="56" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D27" s="26" t="n">
+      <c r="D27" s="30" t="n">
         <v>963.58</v>
       </c>
-      <c r="E27" s="27" t="n">
+      <c r="E27" s="31" t="n">
         <v>0.1238</v>
       </c>
-      <c r="F27" s="27" t="n">
+      <c r="F27" s="31" t="n">
         <v>0.0146</v>
       </c>
-      <c r="G27" s="40" t="n">
+      <c r="G27" s="44" t="n">
         <v>1.2476</v>
       </c>
-      <c r="H27" s="40" t="n">
+      <c r="H27" s="44" t="n">
         <v>1.1847</v>
       </c>
-      <c r="I27" s="40" t="n">
+      <c r="I27" s="44" t="n">
         <v>1.2551</v>
       </c>
-      <c r="J27" s="53" t="n">
+      <c r="J27" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K27" s="26" t="n">
+      <c r="K27" s="30" t="n">
         <v>31533</v>
       </c>
-      <c r="L27" s="54" t="inlineStr">
+      <c r="L27" s="58" t="inlineStr">
         <is>
           <t>MBWAY_NAN</t>
         </is>
@@ -3286,42 +3571,42 @@
       <c r="W27" s="1" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="51" t="inlineStr"/>
-      <c r="B28" s="25" t="inlineStr">
+      <c r="A28" s="55" t="inlineStr"/>
+      <c r="B28" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C28" s="52" t="inlineStr">
+      <c r="C28" s="56" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D28" s="26" t="n">
+      <c r="D28" s="30" t="n">
         <v>1475.02</v>
       </c>
-      <c r="E28" s="27" t="n">
+      <c r="E28" s="31" t="n">
         <v>0.1107</v>
       </c>
-      <c r="F28" s="27" t="n">
+      <c r="F28" s="31" t="n">
         <v>0.0218</v>
       </c>
-      <c r="G28" s="40" t="n">
+      <c r="G28" s="44" t="n">
         <v>0.8149999999999999</v>
       </c>
-      <c r="H28" s="40" t="n">
+      <c r="H28" s="44" t="n">
         <v>1.0597</v>
       </c>
-      <c r="I28" s="40" t="n">
+      <c r="I28" s="44" t="n">
         <v>0.8428</v>
       </c>
-      <c r="J28" s="53" t="n">
+      <c r="J28" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K28" s="26" t="n">
+      <c r="K28" s="30" t="n">
         <v>68291</v>
       </c>
-      <c r="L28" s="54" t="inlineStr">
+      <c r="L28" s="58" t="inlineStr">
         <is>
           <t>MBWAY_PAR</t>
         </is>
@@ -3339,42 +3624,42 @@
       <c r="W28" s="1" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="51" t="inlineStr"/>
-      <c r="B29" s="25" t="inlineStr">
+      <c r="A29" s="55" t="inlineStr"/>
+      <c r="B29" s="29" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C29" s="52" t="inlineStr">
+      <c r="C29" s="56" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D29" s="26" t="n">
+      <c r="D29" s="30" t="n">
         <v>1368.09</v>
       </c>
-      <c r="E29" s="27" t="n">
+      <c r="E29" s="31" t="n">
         <v>0.08749999999999999</v>
       </c>
-      <c r="F29" s="27" t="n">
+      <c r="F29" s="31" t="n">
         <v>0.0194</v>
       </c>
-      <c r="G29" s="40" t="n">
+      <c r="G29" s="44" t="n">
         <v>0.8787</v>
       </c>
-      <c r="H29" s="40" t="n">
+      <c r="H29" s="44" t="n">
         <v>0.8377</v>
       </c>
-      <c r="I29" s="40" t="n">
+      <c r="I29" s="44" t="n">
         <v>0.9454</v>
       </c>
-      <c r="J29" s="53" t="n">
+      <c r="J29" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K29" s="26" t="n">
+      <c r="K29" s="30" t="n">
         <v>21968</v>
       </c>
-      <c r="L29" s="54" t="inlineStr">
+      <c r="L29" s="58" t="inlineStr">
         <is>
           <t>PIGIER_BOR</t>
         </is>
@@ -3392,42 +3677,42 @@
       <c r="W29" s="1" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="51" t="inlineStr"/>
-      <c r="B30" s="25" t="inlineStr">
+      <c r="A30" s="55" t="inlineStr"/>
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C30" s="52" t="inlineStr">
+      <c r="C30" s="56" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D30" s="26" t="n">
+      <c r="D30" s="30" t="n">
         <v>1704.98</v>
       </c>
-      <c r="E30" s="27" t="n">
+      <c r="E30" s="31" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="F30" s="27" t="n">
+      <c r="F30" s="31" t="n">
         <v>0.0233</v>
       </c>
-      <c r="G30" s="40" t="n">
+      <c r="G30" s="44" t="n">
         <v>0.7050999999999999</v>
       </c>
-      <c r="H30" s="40" t="n">
+      <c r="H30" s="44" t="n">
         <v>0.8135</v>
       </c>
-      <c r="I30" s="40" t="n">
+      <c r="I30" s="44" t="n">
         <v>0.7883</v>
       </c>
-      <c r="J30" s="53" t="n">
+      <c r="J30" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K30" s="26" t="n">
+      <c r="K30" s="30" t="n">
         <v>36612</v>
       </c>
-      <c r="L30" s="54" t="inlineStr">
+      <c r="L30" s="58" t="inlineStr">
         <is>
           <t>PIGIER_LYO</t>
         </is>
@@ -3445,42 +3730,42 @@
       <c r="W30" s="1" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="51" t="inlineStr"/>
-      <c r="B31" s="25" t="inlineStr">
+      <c r="A31" s="55" t="inlineStr"/>
+      <c r="B31" s="29" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C31" s="52" t="inlineStr">
+      <c r="C31" s="56" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D31" s="26" t="n">
+      <c r="D31" s="30" t="n">
         <v>1624.68</v>
       </c>
-      <c r="E31" s="27" t="n">
+      <c r="E31" s="31" t="n">
         <v>0.0726</v>
       </c>
-      <c r="F31" s="27" t="n">
+      <c r="F31" s="31" t="n">
         <v>0.0218</v>
       </c>
-      <c r="G31" s="40" t="n">
+      <c r="G31" s="44" t="n">
         <v>0.7399</v>
       </c>
-      <c r="H31" s="40" t="n">
+      <c r="H31" s="44" t="n">
         <v>0.6943</v>
       </c>
-      <c r="I31" s="40" t="n">
+      <c r="I31" s="44" t="n">
         <v>0.8401</v>
       </c>
-      <c r="J31" s="53" t="n">
+      <c r="J31" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K31" s="26" t="n">
+      <c r="K31" s="30" t="n">
         <v>18850</v>
       </c>
-      <c r="L31" s="54" t="inlineStr">
+      <c r="L31" s="58" t="inlineStr">
         <is>
           <t>TUNON_LYO</t>
         </is>
@@ -3498,42 +3783,42 @@
       <c r="W31" s="1" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="51" t="inlineStr"/>
-      <c r="B32" s="25" t="inlineStr">
+      <c r="A32" s="55" t="inlineStr"/>
+      <c r="B32" s="29" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C32" s="52" t="inlineStr">
+      <c r="C32" s="56" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D32" s="26" t="n">
+      <c r="D32" s="30" t="n">
         <v>2192.89</v>
       </c>
-      <c r="E32" s="27" t="n">
+      <c r="E32" s="31" t="n">
         <v>0.06950000000000001</v>
       </c>
-      <c r="F32" s="27" t="n">
+      <c r="F32" s="31" t="n">
         <v>0.0278</v>
       </c>
-      <c r="G32" s="40" t="n">
+      <c r="G32" s="44" t="n">
         <v>0.5482</v>
       </c>
-      <c r="H32" s="40" t="n">
+      <c r="H32" s="44" t="n">
         <v>0.6653</v>
       </c>
-      <c r="I32" s="40" t="n">
+      <c r="I32" s="44" t="n">
         <v>0.6586</v>
       </c>
-      <c r="J32" s="53" t="n">
+      <c r="J32" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="K32" s="26" t="n">
+      <c r="K32" s="30" t="n">
         <v>30240</v>
       </c>
-      <c r="L32" s="54" t="inlineStr">
+      <c r="L32" s="58" t="inlineStr">
         <is>
           <t>TUNON_PAR</t>
         </is>
@@ -3627,21 +3912,21 @@
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="21" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>SYNTHÈSE PAR CAMPUS</t>
         </is>
       </c>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="22" t="n"/>
-      <c r="G36" s="22" t="n"/>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="22" t="n"/>
-      <c r="J36" s="22" t="n"/>
-      <c r="K36" s="22" t="n"/>
-      <c r="L36" s="22" t="n"/>
+      <c r="C36" s="26" t="n"/>
+      <c r="D36" s="26" t="n"/>
+      <c r="E36" s="26" t="n"/>
+      <c r="F36" s="26" t="n"/>
+      <c r="G36" s="26" t="n"/>
+      <c r="H36" s="26" t="n"/>
+      <c r="I36" s="26" t="n"/>
+      <c r="J36" s="26" t="n"/>
+      <c r="K36" s="26" t="n"/>
+      <c r="L36" s="26" t="n"/>
       <c r="M36" s="1" t="n"/>
       <c r="N36" s="1" t="n"/>
       <c r="O36" s="1" t="n"/>
@@ -3680,58 +3965,58 @@
       <c r="W37" s="1" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="47" t="inlineStr"/>
-      <c r="B38" s="48" t="inlineStr">
+      <c r="A38" s="51" t="inlineStr"/>
+      <c r="B38" s="52" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="C38" s="48" t="inlineStr">
+      <c r="C38" s="52" t="inlineStr">
         <is>
           <t>Ville</t>
         </is>
       </c>
-      <c r="D38" s="49" t="inlineStr">
+      <c r="D38" s="53" t="inlineStr">
         <is>
           <t>Effectif</t>
         </is>
       </c>
-      <c r="E38" s="49" t="inlineStr">
+      <c r="E38" s="53" t="inlineStr">
         <is>
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="F38" s="49" t="inlineStr">
+      <c r="F38" s="53" t="inlineStr">
         <is>
           <t>Prix moyen</t>
         </is>
       </c>
-      <c r="G38" s="49" t="inlineStr">
+      <c r="G38" s="53" t="inlineStr">
         <is>
           <t>Part du CA</t>
         </is>
       </c>
-      <c r="H38" s="49" t="inlineStr">
+      <c r="H38" s="53" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="I38" s="47" t="inlineStr">
+      <c r="I38" s="51" t="inlineStr">
         <is>
           <t>Marge</t>
         </is>
       </c>
-      <c r="J38" s="49" t="inlineStr">
+      <c r="J38" s="53" t="inlineStr">
         <is>
           <t>EBITDA par étudiant</t>
         </is>
       </c>
-      <c r="K38" s="49" t="inlineStr">
+      <c r="K38" s="53" t="inlineStr">
         <is>
           <t>Budget acquisition</t>
         </is>
       </c>
-      <c r="L38" s="49" t="inlineStr">
+      <c r="L38" s="53" t="inlineStr">
         <is>
           <t>CAC marginal</t>
         </is>
@@ -3749,42 +4034,42 @@
       <c r="W38" s="1" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="51" t="inlineStr"/>
-      <c r="B39" s="25" t="inlineStr">
+      <c r="A39" s="55" t="inlineStr"/>
+      <c r="B39" s="29" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C39" s="52" t="inlineStr">
+      <c r="C39" s="56" t="inlineStr">
         <is>
           <t>Montpellier</t>
         </is>
       </c>
-      <c r="D39" s="55" t="n">
+      <c r="D39" s="59" t="n">
         <v>122.13</v>
       </c>
-      <c r="E39" s="26" t="n">
+      <c r="E39" s="30" t="n">
         <v>818445.73</v>
       </c>
-      <c r="F39" s="26" t="n">
+      <c r="F39" s="30" t="n">
         <v>6701.29</v>
       </c>
-      <c r="G39" s="27" t="n">
+      <c r="G39" s="31" t="n">
         <v>0.0338</v>
       </c>
-      <c r="H39" s="26" t="n">
+      <c r="H39" s="30" t="n">
         <v>254308.3</v>
       </c>
-      <c r="I39" s="56" t="n">
+      <c r="I39" s="60" t="n">
         <v>0.3107</v>
       </c>
-      <c r="J39" s="26" t="n">
+      <c r="J39" s="30" t="n">
         <v>2082.23</v>
       </c>
-      <c r="K39" s="26" t="n">
+      <c r="K39" s="30" t="n">
         <v>15178</v>
       </c>
-      <c r="L39" s="26" t="n">
+      <c r="L39" s="30" t="n">
         <v>1033.98</v>
       </c>
       <c r="M39" s="1" t="n"/>
@@ -3800,42 +4085,42 @@
       <c r="W39" s="1" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="51" t="inlineStr"/>
-      <c r="B40" s="25" t="inlineStr">
+      <c r="A40" s="55" t="inlineStr"/>
+      <c r="B40" s="29" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C40" s="52" t="inlineStr">
+      <c r="C40" s="56" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D40" s="55" t="n">
+      <c r="D40" s="59" t="n">
         <v>151.32</v>
       </c>
-      <c r="E40" s="26" t="n">
+      <c r="E40" s="30" t="n">
         <v>1067200.79</v>
       </c>
-      <c r="F40" s="26" t="n">
+      <c r="F40" s="30" t="n">
         <v>7052.49</v>
       </c>
-      <c r="G40" s="27" t="n">
+      <c r="G40" s="31" t="n">
         <v>0.044</v>
       </c>
-      <c r="H40" s="26" t="n">
+      <c r="H40" s="30" t="n">
         <v>331184.51</v>
       </c>
-      <c r="I40" s="56" t="n">
+      <c r="I40" s="60" t="n">
         <v>0.3103</v>
       </c>
-      <c r="J40" s="26" t="n">
+      <c r="J40" s="30" t="n">
         <v>2188.6</v>
       </c>
-      <c r="K40" s="26" t="n">
+      <c r="K40" s="30" t="n">
         <v>21760</v>
       </c>
-      <c r="L40" s="26" t="n">
+      <c r="L40" s="30" t="n">
         <v>1216.29</v>
       </c>
       <c r="M40" s="1" t="n"/>
@@ -3851,42 +4136,42 @@
       <c r="W40" s="1" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="51" t="inlineStr"/>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="A41" s="55" t="inlineStr"/>
+      <c r="B41" s="29" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C41" s="52" t="inlineStr">
+      <c r="C41" s="56" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="D41" s="55" t="n">
+      <c r="D41" s="59" t="n">
         <v>122.12</v>
       </c>
-      <c r="E41" s="26" t="n">
+      <c r="E41" s="30" t="n">
         <v>818371.29</v>
       </c>
-      <c r="F41" s="26" t="n">
+      <c r="F41" s="30" t="n">
         <v>6701.28</v>
       </c>
-      <c r="G41" s="27" t="n">
+      <c r="G41" s="31" t="n">
         <v>0.0338</v>
       </c>
-      <c r="H41" s="26" t="n">
+      <c r="H41" s="30" t="n">
         <v>254316.41</v>
       </c>
-      <c r="I41" s="56" t="n">
+      <c r="I41" s="60" t="n">
         <v>0.3108</v>
       </c>
-      <c r="J41" s="26" t="n">
+      <c r="J41" s="30" t="n">
         <v>2082.49</v>
       </c>
-      <c r="K41" s="26" t="n">
+      <c r="K41" s="30" t="n">
         <v>14933</v>
       </c>
-      <c r="L41" s="26" t="n">
+      <c r="L41" s="30" t="n">
         <v>1040.56</v>
       </c>
       <c r="M41" s="1" t="n"/>
@@ -3902,42 +4187,42 @@
       <c r="W41" s="1" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="51" t="inlineStr"/>
-      <c r="B42" s="25" t="inlineStr">
+      <c r="A42" s="55" t="inlineStr"/>
+      <c r="B42" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C42" s="52" t="inlineStr">
+      <c r="C42" s="56" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="D42" s="55" t="n">
+      <c r="D42" s="59" t="n">
         <v>255.09</v>
       </c>
-      <c r="E42" s="26" t="n">
+      <c r="E42" s="30" t="n">
         <v>1844124.54</v>
       </c>
-      <c r="F42" s="26" t="n">
+      <c r="F42" s="30" t="n">
         <v>7229.4</v>
       </c>
-      <c r="G42" s="27" t="n">
+      <c r="G42" s="31" t="n">
         <v>0.0761</v>
       </c>
-      <c r="H42" s="26" t="n">
+      <c r="H42" s="30" t="n">
         <v>602778.74</v>
       </c>
-      <c r="I42" s="56" t="n">
+      <c r="I42" s="60" t="n">
         <v>0.3269</v>
       </c>
-      <c r="J42" s="26" t="n">
+      <c r="J42" s="30" t="n">
         <v>2363.04</v>
       </c>
-      <c r="K42" s="26" t="n">
+      <c r="K42" s="30" t="n">
         <v>25220</v>
       </c>
-      <c r="L42" s="26" t="n">
+      <c r="L42" s="30" t="n">
         <v>978.58</v>
       </c>
       <c r="M42" s="1" t="n"/>
@@ -3953,42 +4238,42 @@
       <c r="W42" s="1" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="51" t="inlineStr"/>
-      <c r="B43" s="25" t="inlineStr">
+      <c r="A43" s="55" t="inlineStr"/>
+      <c r="B43" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C43" s="52" t="inlineStr">
+      <c r="C43" s="56" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D43" s="55" t="n">
+      <c r="D43" s="59" t="n">
         <v>369.35</v>
       </c>
-      <c r="E43" s="26" t="n">
+      <c r="E43" s="30" t="n">
         <v>3048653.48</v>
       </c>
-      <c r="F43" s="26" t="n">
+      <c r="F43" s="30" t="n">
         <v>8254.049999999999</v>
       </c>
-      <c r="G43" s="27" t="n">
+      <c r="G43" s="31" t="n">
         <v>0.1258</v>
       </c>
-      <c r="H43" s="26" t="n">
+      <c r="H43" s="30" t="n">
         <v>985765.87</v>
       </c>
-      <c r="I43" s="56" t="n">
+      <c r="I43" s="60" t="n">
         <v>0.3233</v>
       </c>
-      <c r="J43" s="26" t="n">
+      <c r="J43" s="30" t="n">
         <v>2668.9</v>
       </c>
-      <c r="K43" s="26" t="n">
+      <c r="K43" s="30" t="n">
         <v>60800</v>
       </c>
-      <c r="L43" s="26" t="n">
+      <c r="L43" s="30" t="n">
         <v>1540.33</v>
       </c>
       <c r="M43" s="1" t="n"/>
@@ -4004,42 +4289,42 @@
       <c r="W43" s="1" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="51" t="inlineStr"/>
-      <c r="B44" s="25" t="inlineStr">
+      <c r="A44" s="55" t="inlineStr"/>
+      <c r="B44" s="29" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C44" s="52" t="inlineStr">
+      <c r="C44" s="56" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="D44" s="55" t="n">
+      <c r="D44" s="59" t="n">
         <v>241.48</v>
       </c>
-      <c r="E44" s="26" t="n">
+      <c r="E44" s="30" t="n">
         <v>1709754.85</v>
       </c>
-      <c r="F44" s="26" t="n">
+      <c r="F44" s="30" t="n">
         <v>7080.28</v>
       </c>
-      <c r="G44" s="27" t="n">
+      <c r="G44" s="31" t="n">
         <v>0.0706</v>
       </c>
-      <c r="H44" s="26" t="n">
+      <c r="H44" s="30" t="n">
         <v>560009.03</v>
       </c>
-      <c r="I44" s="56" t="n">
+      <c r="I44" s="60" t="n">
         <v>0.3275</v>
       </c>
-      <c r="J44" s="26" t="n">
+      <c r="J44" s="30" t="n">
         <v>2319.06</v>
       </c>
-      <c r="K44" s="26" t="n">
+      <c r="K44" s="30" t="n">
         <v>22083</v>
       </c>
-      <c r="L44" s="26" t="n">
+      <c r="L44" s="30" t="n">
         <v>919.03</v>
       </c>
       <c r="M44" s="1" t="n"/>
@@ -4055,42 +4340,42 @@
       <c r="W44" s="1" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="51" t="inlineStr"/>
-      <c r="B45" s="25" t="inlineStr">
+      <c r="A45" s="55" t="inlineStr"/>
+      <c r="B45" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C45" s="52" t="inlineStr">
+      <c r="C45" s="56" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D45" s="55" t="n">
+      <c r="D45" s="59" t="n">
         <v>260.41</v>
       </c>
-      <c r="E45" s="26" t="n">
+      <c r="E45" s="30" t="n">
         <v>1863775.69</v>
       </c>
-      <c r="F45" s="26" t="n">
+      <c r="F45" s="30" t="n">
         <v>7157.03</v>
       </c>
-      <c r="G45" s="27" t="n">
+      <c r="G45" s="31" t="n">
         <v>0.0769</v>
       </c>
-      <c r="H45" s="26" t="n">
+      <c r="H45" s="30" t="n">
         <v>625402.3</v>
       </c>
-      <c r="I45" s="56" t="n">
+      <c r="I45" s="60" t="n">
         <v>0.3356</v>
       </c>
-      <c r="J45" s="26" t="n">
+      <c r="J45" s="30" t="n">
         <v>2401.59</v>
       </c>
-      <c r="K45" s="26" t="n">
+      <c r="K45" s="30" t="n">
         <v>24923</v>
       </c>
-      <c r="L45" s="26" t="n">
+      <c r="L45" s="30" t="n">
         <v>889.59</v>
       </c>
       <c r="M45" s="1" t="n"/>
@@ -4106,42 +4391,42 @@
       <c r="W45" s="1" t="n"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="51" t="inlineStr"/>
-      <c r="B46" s="25" t="inlineStr">
+      <c r="A46" s="55" t="inlineStr"/>
+      <c r="B46" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C46" s="52" t="inlineStr">
+      <c r="C46" s="56" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D46" s="55" t="n">
+      <c r="D46" s="59" t="n">
         <v>338.5</v>
       </c>
-      <c r="E46" s="26" t="n">
+      <c r="E46" s="30" t="n">
         <v>2620797.34</v>
       </c>
-      <c r="F46" s="26" t="n">
+      <c r="F46" s="30" t="n">
         <v>7742.43</v>
       </c>
-      <c r="G46" s="27" t="n">
+      <c r="G46" s="31" t="n">
         <v>0.1082</v>
       </c>
-      <c r="H46" s="26" t="n">
+      <c r="H46" s="30" t="n">
         <v>876442.71</v>
       </c>
-      <c r="I46" s="56" t="n">
+      <c r="I46" s="60" t="n">
         <v>0.3344</v>
       </c>
-      <c r="J46" s="26" t="n">
+      <c r="J46" s="30" t="n">
         <v>2589.21</v>
       </c>
-      <c r="K46" s="26" t="n">
+      <c r="K46" s="30" t="n">
         <v>41783</v>
       </c>
-      <c r="L46" s="26" t="n">
+      <c r="L46" s="30" t="n">
         <v>1101.6</v>
       </c>
       <c r="M46" s="1" t="n"/>
@@ -4157,42 +4442,42 @@
       <c r="W46" s="1" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="51" t="inlineStr"/>
-      <c r="B47" s="25" t="inlineStr">
+      <c r="A47" s="55" t="inlineStr"/>
+      <c r="B47" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C47" s="52" t="inlineStr">
+      <c r="C47" s="56" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D47" s="55" t="n">
+      <c r="D47" s="59" t="n">
         <v>307.34</v>
       </c>
-      <c r="E47" s="26" t="n">
+      <c r="E47" s="30" t="n">
         <v>2267018.63</v>
       </c>
-      <c r="F47" s="26" t="n">
+      <c r="F47" s="30" t="n">
         <v>7376.18</v>
       </c>
-      <c r="G47" s="27" t="n">
+      <c r="G47" s="31" t="n">
         <v>0.0936</v>
       </c>
-      <c r="H47" s="26" t="n">
+      <c r="H47" s="30" t="n">
         <v>763702.73</v>
       </c>
-      <c r="I47" s="56" t="n">
+      <c r="I47" s="60" t="n">
         <v>0.3369</v>
       </c>
-      <c r="J47" s="26" t="n">
+      <c r="J47" s="30" t="n">
         <v>2484.86</v>
       </c>
-      <c r="K47" s="26" t="n">
+      <c r="K47" s="30" t="n">
         <v>31533</v>
       </c>
-      <c r="L47" s="26" t="n">
+      <c r="L47" s="30" t="n">
         <v>963.58</v>
       </c>
       <c r="M47" s="1" t="n"/>
@@ -4208,42 +4493,42 @@
       <c r="W47" s="1" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="51" t="inlineStr"/>
-      <c r="B48" s="25" t="inlineStr">
+      <c r="A48" s="55" t="inlineStr"/>
+      <c r="B48" s="29" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C48" s="52" t="inlineStr">
+      <c r="C48" s="56" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D48" s="55" t="n">
+      <c r="D48" s="59" t="n">
         <v>398.78</v>
       </c>
-      <c r="E48" s="26" t="n">
+      <c r="E48" s="30" t="n">
         <v>3292150.8</v>
       </c>
-      <c r="F48" s="26" t="n">
+      <c r="F48" s="30" t="n">
         <v>8255.51</v>
       </c>
-      <c r="G48" s="27" t="n">
+      <c r="G48" s="31" t="n">
         <v>0.1359</v>
       </c>
-      <c r="H48" s="26" t="n">
+      <c r="H48" s="30" t="n">
         <v>1096393.82</v>
       </c>
-      <c r="I48" s="56" t="n">
+      <c r="I48" s="60" t="n">
         <v>0.333</v>
       </c>
-      <c r="J48" s="26" t="n">
+      <c r="J48" s="30" t="n">
         <v>2749.35</v>
       </c>
-      <c r="K48" s="26" t="n">
+      <c r="K48" s="30" t="n">
         <v>68291</v>
       </c>
-      <c r="L48" s="26" t="n">
+      <c r="L48" s="30" t="n">
         <v>1475.02</v>
       </c>
       <c r="M48" s="1" t="n"/>
@@ -4259,42 +4544,42 @@
       <c r="W48" s="1" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="51" t="inlineStr"/>
-      <c r="B49" s="25" t="inlineStr">
+      <c r="A49" s="55" t="inlineStr"/>
+      <c r="B49" s="29" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C49" s="52" t="inlineStr">
+      <c r="C49" s="56" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D49" s="55" t="n">
+      <c r="D49" s="59" t="n">
         <v>184.72</v>
       </c>
-      <c r="E49" s="26" t="n">
+      <c r="E49" s="30" t="n">
         <v>1191512.54</v>
       </c>
-      <c r="F49" s="26" t="n">
+      <c r="F49" s="30" t="n">
         <v>6450.49</v>
       </c>
-      <c r="G49" s="27" t="n">
+      <c r="G49" s="31" t="n">
         <v>0.0492</v>
       </c>
-      <c r="H49" s="26" t="n">
+      <c r="H49" s="30" t="n">
         <v>455099.2</v>
       </c>
-      <c r="I49" s="56" t="n">
+      <c r="I49" s="60" t="n">
         <v>0.382</v>
       </c>
-      <c r="J49" s="26" t="n">
+      <c r="J49" s="30" t="n">
         <v>2463.77</v>
       </c>
-      <c r="K49" s="26" t="n">
+      <c r="K49" s="30" t="n">
         <v>21968</v>
       </c>
-      <c r="L49" s="26" t="n">
+      <c r="L49" s="30" t="n">
         <v>1368.09</v>
       </c>
       <c r="M49" s="1" t="n"/>
@@ -4310,42 +4595,42 @@
       <c r="W49" s="1" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="51" t="inlineStr"/>
-      <c r="B50" s="25" t="inlineStr">
+      <c r="A50" s="55" t="inlineStr"/>
+      <c r="B50" s="29" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C50" s="52" t="inlineStr">
+      <c r="C50" s="56" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D50" s="55" t="n">
+      <c r="D50" s="59" t="n">
         <v>236.95</v>
       </c>
-      <c r="E50" s="26" t="n">
+      <c r="E50" s="30" t="n">
         <v>1653869.91</v>
       </c>
-      <c r="F50" s="26" t="n">
+      <c r="F50" s="30" t="n">
         <v>6979.9</v>
       </c>
-      <c r="G50" s="27" t="n">
+      <c r="G50" s="31" t="n">
         <v>0.0683</v>
       </c>
-      <c r="H50" s="26" t="n">
+      <c r="H50" s="30" t="n">
         <v>626670.52</v>
       </c>
-      <c r="I50" s="56" t="n">
+      <c r="I50" s="60" t="n">
         <v>0.3789</v>
       </c>
-      <c r="J50" s="26" t="n">
+      <c r="J50" s="30" t="n">
         <v>2644.77</v>
       </c>
-      <c r="K50" s="26" t="n">
+      <c r="K50" s="30" t="n">
         <v>36612</v>
       </c>
-      <c r="L50" s="26" t="n">
+      <c r="L50" s="30" t="n">
         <v>1704.98</v>
       </c>
       <c r="M50" s="1" t="n"/>
@@ -4361,42 +4646,42 @@
       <c r="W50" s="1" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="51" t="inlineStr"/>
-      <c r="B51" s="25" t="inlineStr">
+      <c r="A51" s="55" t="inlineStr"/>
+      <c r="B51" s="29" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C51" s="52" t="inlineStr">
+      <c r="C51" s="56" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D51" s="55" t="n">
+      <c r="D51" s="59" t="n">
         <v>121.86</v>
       </c>
-      <c r="E51" s="26" t="n">
+      <c r="E51" s="30" t="n">
         <v>902399.37</v>
       </c>
-      <c r="F51" s="26" t="n">
+      <c r="F51" s="30" t="n">
         <v>7405.22</v>
       </c>
-      <c r="G51" s="27" t="n">
+      <c r="G51" s="31" t="n">
         <v>0.0372</v>
       </c>
-      <c r="H51" s="26" t="n">
+      <c r="H51" s="30" t="n">
         <v>178759.19</v>
       </c>
-      <c r="I51" s="56" t="n">
+      <c r="I51" s="60" t="n">
         <v>0.1981</v>
       </c>
-      <c r="J51" s="26" t="n">
+      <c r="J51" s="30" t="n">
         <v>1466.92</v>
       </c>
-      <c r="K51" s="26" t="n">
+      <c r="K51" s="30" t="n">
         <v>18850</v>
       </c>
-      <c r="L51" s="26" t="n">
+      <c r="L51" s="30" t="n">
         <v>1624.68</v>
       </c>
       <c r="M51" s="1" t="n"/>
@@ -4412,42 +4697,42 @@
       <c r="W51" s="1" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="51" t="inlineStr"/>
-      <c r="B52" s="25" t="inlineStr">
+      <c r="A52" s="55" t="inlineStr"/>
+      <c r="B52" s="29" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C52" s="52" t="inlineStr">
+      <c r="C52" s="56" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D52" s="55" t="n">
+      <c r="D52" s="59" t="n">
         <v>143.56</v>
       </c>
-      <c r="E52" s="26" t="n">
+      <c r="E52" s="30" t="n">
         <v>1133628.58</v>
       </c>
-      <c r="F52" s="26" t="n">
+      <c r="F52" s="30" t="n">
         <v>7896.53</v>
       </c>
-      <c r="G52" s="27" t="n">
+      <c r="G52" s="31" t="n">
         <v>0.0468</v>
       </c>
-      <c r="H52" s="26" t="n">
+      <c r="H52" s="30" t="n">
         <v>220510.28</v>
       </c>
-      <c r="I52" s="56" t="n">
+      <c r="I52" s="60" t="n">
         <v>0.1945</v>
       </c>
-      <c r="J52" s="26" t="n">
+      <c r="J52" s="30" t="n">
         <v>1536.01</v>
       </c>
-      <c r="K52" s="26" t="n">
+      <c r="K52" s="30" t="n">
         <v>30240</v>
       </c>
-      <c r="L52" s="26" t="n">
+      <c r="L52" s="30" t="n">
         <v>2192.89</v>
       </c>
       <c r="M52" s="1" t="n"/>
@@ -4463,38 +4748,38 @@
       <c r="W52" s="1" t="n"/>
     </row>
     <row r="53" ht="17" customHeight="1">
-      <c r="A53" s="57" t="n"/>
-      <c r="B53" s="58" t="inlineStr">
+      <c r="A53" s="61" t="n"/>
+      <c r="B53" s="62" t="inlineStr">
         <is>
           <t>Total campus</t>
         </is>
       </c>
-      <c r="C53" s="57" t="n"/>
-      <c r="D53" s="59" t="n">
+      <c r="C53" s="61" t="n"/>
+      <c r="D53" s="63" t="n">
         <v>3253.62</v>
       </c>
-      <c r="E53" s="60" t="n">
+      <c r="E53" s="64" t="n">
         <v>24231703.55</v>
       </c>
-      <c r="F53" s="60" t="n">
+      <c r="F53" s="64" t="n">
         <v>7447.62</v>
       </c>
-      <c r="G53" s="61" t="n">
+      <c r="G53" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="H53" s="60" t="n">
+      <c r="H53" s="64" t="n">
         <v>7831343.62</v>
       </c>
-      <c r="I53" s="62" t="n">
+      <c r="I53" s="66" t="n">
         <v>0.3232</v>
       </c>
-      <c r="J53" s="60" t="n">
+      <c r="J53" s="64" t="n">
         <v>2406.97</v>
       </c>
-      <c r="K53" s="60" t="n">
+      <c r="K53" s="64" t="n">
         <v>434174</v>
       </c>
-      <c r="L53" s="57" t="n"/>
+      <c r="L53" s="61" t="n"/>
       <c r="M53" s="1" t="n"/>
       <c r="N53" s="1" t="n"/>
       <c r="O53" s="1" t="n"/>
@@ -4508,24 +4793,24 @@
       <c r="W53" s="1" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="63" t="n"/>
-      <c r="B54" s="64" t="inlineStr">
+      <c r="A54" s="67" t="n"/>
+      <c r="B54" s="68" t="inlineStr">
         <is>
           <t>Siège et holding</t>
         </is>
       </c>
-      <c r="C54" s="63" t="n"/>
-      <c r="D54" s="63" t="n"/>
-      <c r="E54" s="63" t="n"/>
-      <c r="F54" s="63" t="n"/>
-      <c r="G54" s="63" t="n"/>
-      <c r="H54" s="65" t="n">
+      <c r="C54" s="67" t="n"/>
+      <c r="D54" s="67" t="n"/>
+      <c r="E54" s="67" t="n"/>
+      <c r="F54" s="67" t="n"/>
+      <c r="G54" s="67" t="n"/>
+      <c r="H54" s="69" t="n">
         <v>-3719839.98</v>
       </c>
-      <c r="I54" s="63" t="n"/>
-      <c r="J54" s="63" t="n"/>
-      <c r="K54" s="63" t="n"/>
-      <c r="L54" s="63" t="n"/>
+      <c r="I54" s="67" t="n"/>
+      <c r="J54" s="67" t="n"/>
+      <c r="K54" s="67" t="n"/>
+      <c r="L54" s="67" t="n"/>
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="n"/>
       <c r="O54" s="1" t="n"/>
@@ -4539,38 +4824,38 @@
       <c r="W54" s="1" t="n"/>
     </row>
     <row r="55" ht="19" customHeight="1">
-      <c r="A55" s="66" t="n"/>
-      <c r="B55" s="67" t="inlineStr">
+      <c r="A55" s="70" t="n"/>
+      <c r="B55" s="71" t="inlineStr">
         <is>
           <t>Groupe</t>
         </is>
       </c>
-      <c r="C55" s="66" t="n"/>
-      <c r="D55" s="68" t="n">
+      <c r="C55" s="70" t="n"/>
+      <c r="D55" s="72" t="n">
         <v>3253.62</v>
       </c>
-      <c r="E55" s="69" t="n">
+      <c r="E55" s="73" t="n">
         <v>24231703.55</v>
       </c>
-      <c r="F55" s="69" t="n">
+      <c r="F55" s="73" t="n">
         <v>7447.62</v>
       </c>
-      <c r="G55" s="70" t="n">
+      <c r="G55" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="H55" s="69" t="n">
+      <c r="H55" s="73" t="n">
         <v>4111503.64</v>
       </c>
-      <c r="I55" s="71" t="n">
+      <c r="I55" s="75" t="n">
         <v>0.1697</v>
       </c>
-      <c r="J55" s="69" t="n">
+      <c r="J55" s="73" t="n">
         <v>1263.67</v>
       </c>
-      <c r="K55" s="69" t="n">
+      <c r="K55" s="73" t="n">
         <v>434174</v>
       </c>
-      <c r="L55" s="66" t="n"/>
+      <c r="L55" s="70" t="n"/>
       <c r="M55" s="1" t="n"/>
       <c r="N55" s="1" t="n"/>
       <c r="O55" s="1" t="n"/>
@@ -4610,7 +4895,7 @@
     </row>
     <row r="57" ht="12" customHeight="1">
       <c r="A57" s="1" t="n"/>
-      <c r="B57" s="44" t="inlineStr">
+      <c r="B57" s="48" t="inlineStr">
         <is>
           <t>Source : Tagetik TGK_MSSQL_07, scénario 2027BUD_V1.</t>
         </is>

</xml_diff>

<commit_message>
Cadrage : le graphique montre le CA et l'EBITDA, plus un graphe de marge
Graphique 1 (H5) : colonnes groupees chiffre d'affaires et EBITDA sur quatre
exercices, meme axe en euros -- pas de second axe -- avec l'objectif EBITDA en
ligne rouge tiretee. La colonne 2027 de chaque serie est dans une teinte
distincte : ce n'est pas un realise.

Graphique 2 (H31) : la marge EBITDA, seule chose que l'axe en euros ne peut pas
montrer. 15,3 % en 2024, 25,2 % en 2027 construit.

Etiquettes en millions a une decimale : en euros pleins, huit etiquettes sur
10 cm se chevauchent.

Zone de donnees P4:T9, hors zone d'impression.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/CAD_PIL_MEP.xlsx
+++ b/eduservices/CAD_PIL_MEP.xlsx
@@ -311,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -343,6 +343,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -609,7 +612,7 @@
                 </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:rPr>
-              <a:t>EBITDA : réel 2024-2026 et budget 2027</a:t>
+              <a:t>Chiffre d'affaires et EBITDA — réel 2024-2026, budget 2027</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -618,7 +621,7 @@
     <plotArea>
       <barChart>
         <barDir val="col"/>
-        <grouping val="stacked"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -629,12 +632,23 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="1F3B57"/>
+              <a:srgbClr val="9DC3E6"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="C9DEF2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
               <f>'Cadrage'!$P$6:$P$9</f>
@@ -656,12 +670,23 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="2E75B6"/>
+              <a:srgbClr val="1F3B57"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
               <f>'Cadrage'!$P$6:$P$9</f>
@@ -674,12 +699,12 @@
           </val>
         </ser>
         <dLbls>
-          <numFmt formatCode="#,##0"/>
+          <numFmt formatCode="#,##0.0,,&quot; M€&quot;"/>
           <txPr>
             <a:bodyPr/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="800">
+                <a:defRPr sz="700">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -689,7 +714,7 @@
               <a:r>
                 <a:t/>
               </a:r>
-              <a:endParaRPr sz="800">
+              <a:endParaRPr sz="700">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -700,7 +725,7 @@
           <showVal val="1"/>
         </dLbls>
         <gapWidth val="60"/>
-        <overlap val="100"/>
+        <overlap val="-15"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -777,6 +802,140 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Marge EBITDA</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cadrage'!T5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3B57"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <cat>
+            <numRef>
+              <f>'Cadrage'!$P$6:$P$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cadrage'!$T$6:$T$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="0.0%"/>
+          <txPr>
+            <a:bodyPr/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="800">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="90"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -786,7 +945,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3744000" cy="2556000"/>
+    <ext cx="3744000" cy="2664000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -796,6 +955,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3744000" cy="1655999"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1093,7 +1274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S46"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1110,9 +1291,10 @@
     <col width="2" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1">
@@ -1135,6 +1317,7 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -1164,6 +1347,7 @@
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
+      <c r="T2" s="1" t="n"/>
     </row>
     <row r="3" ht="6" customHeight="1">
       <c r="A3" s="1" t="n"/>
@@ -1185,6 +1369,7 @@
       <c r="Q3" s="1" t="n"/>
       <c r="R3" s="1" t="n"/>
       <c r="S3" s="1" t="n"/>
+      <c r="T3" s="1" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
       <c r="A4" s="1" t="n"/>
@@ -1204,12 +1389,13 @@
       <c r="O4" s="1" t="n"/>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Données du graphique</t>
+          <t>Données des graphiques</t>
         </is>
       </c>
       <c r="Q4" s="1" t="n"/>
       <c r="R4" s="1" t="n"/>
       <c r="S4" s="1" t="n"/>
+      <c r="T4" s="1" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="1" t="n"/>
@@ -1248,17 +1434,22 @@
       </c>
       <c r="Q5" s="10" t="inlineStr">
         <is>
-          <t>Réel</t>
+          <t>Chiffre d'affaires</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
-          <t>Budget 2027</t>
+          <t>EBITDA</t>
         </is>
       </c>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>Objectif</t>
+          <t>Objectif EBITDA</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>Marge EBITDA</t>
         </is>
       </c>
     </row>
@@ -1282,32 +1473,37 @@
         <v>2024</v>
       </c>
       <c r="Q6" s="12" t="n">
+        <v>20567210</v>
+      </c>
+      <c r="R6" s="12" t="n">
         <v>3151035</v>
       </c>
-      <c r="R6" s="1" t="n"/>
       <c r="S6" s="12" t="n">
         <v>4095766.36</v>
       </c>
+      <c r="T6" s="13" t="n">
+        <v>0.1532</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="n"/>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Objectif EBITDA 2027</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>EBITDA construit</t>
         </is>
       </c>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Écart à l'objectif</t>
         </is>
       </c>
-      <c r="F7" s="16" t="n"/>
+      <c r="F7" s="17" t="n"/>
       <c r="G7" s="1" t="n"/>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
@@ -1321,26 +1517,31 @@
         <v>2025</v>
       </c>
       <c r="Q7" s="12" t="n">
+        <v>21758770</v>
+      </c>
+      <c r="R7" s="12" t="n">
         <v>3467768</v>
       </c>
-      <c r="R7" s="1" t="n"/>
       <c r="S7" s="12" t="n">
         <v>4095766.36</v>
       </c>
+      <c r="T7" s="13" t="n">
+        <v>0.1594</v>
+      </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="18" t="n">
         <v>4095766.36</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>6744302.91</v>
       </c>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="18" t="n">
+      <c r="D8" s="20" t="n"/>
+      <c r="E8" s="19" t="n">
         <v>2648536.55</v>
       </c>
-      <c r="F8" s="20" t="n"/>
+      <c r="F8" s="21" t="n"/>
       <c r="G8" s="1" t="n"/>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
@@ -1354,32 +1555,37 @@
         <v>2026</v>
       </c>
       <c r="Q8" s="12" t="n">
+        <v>23098985</v>
+      </c>
+      <c r="R8" s="12" t="n">
         <v>3845790</v>
       </c>
-      <c r="R8" s="1" t="n"/>
       <c r="S8" s="12" t="n">
         <v>4095766.36</v>
       </c>
+      <c r="T8" s="13" t="n">
+        <v>0.1665</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>2026 : 3 845 790 €</t>
         </is>
       </c>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>marge 25,2 %</t>
         </is>
       </c>
-      <c r="D9" s="23" t="n"/>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>objectif dépassé</t>
         </is>
       </c>
-      <c r="F9" s="24" t="n"/>
+      <c r="F9" s="25" t="n"/>
       <c r="G9" s="1" t="n"/>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
@@ -1392,25 +1598,30 @@
       <c r="P9" s="11" t="n">
         <v>2027</v>
       </c>
-      <c r="Q9" s="1" t="n"/>
+      <c r="Q9" s="12" t="n">
+        <v>26814168.68</v>
+      </c>
       <c r="R9" s="12" t="n">
         <v>6744302.91</v>
       </c>
       <c r="S9" s="12" t="n">
         <v>4095766.36</v>
       </c>
+      <c r="T9" s="13" t="n">
+        <v>0.2515</v>
+      </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>RÉCONCILIATION 2026 / 2027</t>
         </is>
       </c>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="26" t="n"/>
-      <c r="F10" s="26" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="27" t="n"/>
+      <c r="E10" s="27" t="n"/>
+      <c r="F10" s="27" t="n"/>
       <c r="G10" s="1" t="n"/>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
@@ -1424,30 +1635,31 @@
       <c r="Q10" s="1" t="n"/>
       <c r="R10" s="1" t="n"/>
       <c r="S10" s="1" t="n"/>
+      <c r="T10" s="1" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
         <is>
           <t>Réel 2026</t>
         </is>
       </c>
-      <c r="D11" s="28" t="inlineStr">
+      <c r="D11" s="29" t="inlineStr">
         <is>
           <t>Budget 2027</t>
         </is>
       </c>
-      <c r="E11" s="28" t="inlineStr">
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>Écart</t>
         </is>
       </c>
-      <c r="F11" s="28" t="inlineStr">
+      <c r="F11" s="29" t="inlineStr">
         <is>
           <t>Écart %</t>
         </is>
@@ -1465,24 +1677,25 @@
       <c r="Q11" s="1" t="n"/>
       <c r="R11" s="1" t="n"/>
       <c r="S11" s="1" t="n"/>
+      <c r="T11" s="1" t="n"/>
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="C12" s="30" t="n">
+      <c r="C12" s="31" t="n">
         <v>23098985</v>
       </c>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="31" t="n">
         <v>26814168.68</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="31" t="n">
         <v>3715183.68</v>
       </c>
-      <c r="F12" s="31" t="n">
+      <c r="F12" s="32" t="n">
         <v>0.1608</v>
       </c>
       <c r="G12" s="1" t="n"/>
@@ -1498,24 +1711,25 @@
       <c r="Q12" s="1" t="n"/>
       <c r="R12" s="1" t="n"/>
       <c r="S12" s="1" t="n"/>
+      <c r="T12" s="1" t="n"/>
     </row>
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="32" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C13" s="33" t="n">
+      <c r="C13" s="34" t="n">
         <v>3845790.01</v>
       </c>
-      <c r="D13" s="33" t="n">
+      <c r="D13" s="34" t="n">
         <v>6744302.91</v>
       </c>
-      <c r="E13" s="33" t="n">
+      <c r="E13" s="34" t="n">
         <v>2898512.9</v>
       </c>
-      <c r="F13" s="34" t="n">
+      <c r="F13" s="35" t="n">
         <v>0.7537</v>
       </c>
       <c r="G13" s="1" t="n"/>
@@ -1531,24 +1745,25 @@
       <c r="Q13" s="1" t="n"/>
       <c r="R13" s="1" t="n"/>
       <c r="S13" s="1" t="n"/>
+      <c r="T13" s="1" t="n"/>
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Marge EBITDA</t>
         </is>
       </c>
-      <c r="C14" s="31" t="n">
+      <c r="C14" s="32" t="n">
         <v>0.1665</v>
       </c>
-      <c r="D14" s="31" t="n">
+      <c r="D14" s="32" t="n">
         <v>0.2515</v>
       </c>
-      <c r="E14" s="31" t="n">
+      <c r="E14" s="32" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="F14" s="35" t="n"/>
+      <c r="F14" s="36" t="n"/>
       <c r="G14" s="1" t="n"/>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
@@ -1562,24 +1777,25 @@
       <c r="Q14" s="1" t="n"/>
       <c r="R14" s="1" t="n"/>
       <c r="S14" s="1" t="n"/>
+      <c r="T14" s="1" t="n"/>
     </row>
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Effectif moyen</t>
         </is>
       </c>
-      <c r="C15" s="36" t="n">
+      <c r="C15" s="37" t="n">
         <v>3114</v>
       </c>
-      <c r="D15" s="36" t="n">
+      <c r="D15" s="37" t="n">
         <v>3473.67</v>
       </c>
-      <c r="E15" s="36" t="n">
+      <c r="E15" s="37" t="n">
         <v>359.67</v>
       </c>
-      <c r="F15" s="31" t="n">
+      <c r="F15" s="32" t="n">
         <v>0.1155</v>
       </c>
       <c r="G15" s="1" t="n"/>
@@ -1595,6 +1811,7 @@
       <c r="Q15" s="1" t="n"/>
       <c r="R15" s="1" t="n"/>
       <c r="S15" s="1" t="n"/>
+      <c r="T15" s="1" t="n"/>
     </row>
     <row r="16" ht="12" customHeight="1">
       <c r="A16" s="1" t="n"/>
@@ -1616,6 +1833,7 @@
       <c r="Q16" s="1" t="n"/>
       <c r="R16" s="1" t="n"/>
       <c r="S16" s="1" t="n"/>
+      <c r="T16" s="1" t="n"/>
     </row>
     <row r="17" ht="6" customHeight="1">
       <c r="A17" s="1" t="n"/>
@@ -1637,18 +1855,19 @@
       <c r="Q17" s="1" t="n"/>
       <c r="R17" s="1" t="n"/>
       <c r="S17" s="1" t="n"/>
+      <c r="T17" s="1" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="25" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>HYPOTHÈSES DE CONSTRUCTION</t>
         </is>
       </c>
-      <c r="C18" s="26" t="n"/>
-      <c r="D18" s="26" t="n"/>
-      <c r="E18" s="26" t="n"/>
-      <c r="F18" s="26" t="n"/>
+      <c r="C18" s="27" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="27" t="n"/>
       <c r="G18" s="1" t="n"/>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="1" t="n"/>
@@ -1662,30 +1881,31 @@
       <c r="Q18" s="1" t="n"/>
       <c r="R18" s="1" t="n"/>
       <c r="S18" s="1" t="n"/>
+      <c r="T18" s="1" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="1" t="n"/>
-      <c r="B19" s="27" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>Levier</t>
         </is>
       </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="C19" s="38" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="D19" s="37" t="inlineStr">
+      <c r="D19" s="38" t="inlineStr">
         <is>
           <t>Optimiste</t>
         </is>
       </c>
-      <c r="E19" s="37" t="inlineStr">
+      <c r="E19" s="38" t="inlineStr">
         <is>
           <t>Prudent</t>
         </is>
       </c>
-      <c r="F19" s="38" t="inlineStr">
+      <c r="F19" s="39" t="inlineStr">
         <is>
           <t>Retenu</t>
         </is>
@@ -1703,6 +1923,7 @@
       <c r="Q19" s="1" t="n"/>
       <c r="R19" s="1" t="n"/>
       <c r="S19" s="1" t="n"/>
+      <c r="T19" s="1" t="n"/>
     </row>
     <row r="20" ht="6" customHeight="1">
       <c r="A20" s="1" t="n"/>
@@ -1724,27 +1945,28 @@
       <c r="Q20" s="1" t="n"/>
       <c r="R20" s="1" t="n"/>
       <c r="S20" s="1" t="n"/>
+      <c r="T20" s="1" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="1" t="n"/>
-      <c r="B21" s="39" t="inlineStr">
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>Croissance</t>
         </is>
       </c>
-      <c r="C21" s="40" t="n"/>
-      <c r="D21" s="40" t="n"/>
-      <c r="E21" s="40" t="n"/>
-      <c r="F21" s="40" t="n"/>
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="41" t="n"/>
       <c r="G21" s="1" t="n"/>
       <c r="H21" s="1" t="n"/>
       <c r="I21" s="1" t="n"/>
-      <c r="J21" s="25" t="inlineStr">
+      <c r="J21" s="26" t="inlineStr">
         <is>
           <t>COEFFICIENTS DE PRIX</t>
         </is>
       </c>
-      <c r="K21" s="26" t="n"/>
+      <c r="K21" s="27" t="n"/>
       <c r="L21" s="1" t="n"/>
       <c r="M21" s="1" t="n"/>
       <c r="N21" s="1" t="n"/>
@@ -1753,21 +1975,22 @@
       <c r="Q21" s="1" t="n"/>
       <c r="R21" s="1" t="n"/>
       <c r="S21" s="1" t="n"/>
+      <c r="T21" s="1" t="n"/>
     </row>
     <row r="22" ht="9" customHeight="1">
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="1" t="n"/>
-      <c r="C22" s="41" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="D22" s="41" t="inlineStr">
+      <c r="D22" s="42" t="inlineStr">
         <is>
           <t>Optimiste</t>
         </is>
       </c>
-      <c r="E22" s="41" t="inlineStr">
+      <c r="E22" s="42" t="inlineStr">
         <is>
           <t>Prudent</t>
         </is>
@@ -1786,35 +2009,36 @@
       <c r="Q22" s="1" t="n"/>
       <c r="R22" s="1" t="n"/>
       <c r="S22" s="1" t="n"/>
+      <c r="T22" s="1" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>Variation du budget d'acquisition</t>
         </is>
       </c>
-      <c r="C23" s="42" t="n">
+      <c r="C23" s="43" t="n">
         <v>0.08</v>
       </c>
-      <c r="D23" s="42" t="n">
+      <c r="D23" s="43" t="n">
         <v>0.15</v>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E23" s="43" t="n">
         <v>-0.05</v>
       </c>
-      <c r="F23" s="43" t="n">
+      <c r="F23" s="44" t="n">
         <v>0.15</v>
       </c>
       <c r="G23" s="1" t="n"/>
       <c r="H23" s="1" t="n"/>
       <c r="I23" s="1" t="n"/>
-      <c r="J23" s="27" t="inlineStr">
+      <c r="J23" s="28" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="K23" s="37" t="inlineStr">
+      <c r="K23" s="38" t="inlineStr">
         <is>
           <t>Coeff.</t>
         </is>
@@ -1827,35 +2051,36 @@
       <c r="Q23" s="1" t="n"/>
       <c r="R23" s="1" t="n"/>
       <c r="S23" s="1" t="n"/>
+      <c r="T23" s="1" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>Variation du budget de marque</t>
         </is>
       </c>
-      <c r="C24" s="42" t="n">
+      <c r="C24" s="43" t="n">
         <v>0.1</v>
       </c>
-      <c r="D24" s="42" t="n">
+      <c r="D24" s="43" t="n">
         <v>0.15</v>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E24" s="43" t="n">
         <v>-0.05</v>
       </c>
-      <c r="F24" s="43" t="n">
+      <c r="F24" s="44" t="n">
         <v>0.15</v>
       </c>
       <c r="G24" s="1" t="n"/>
       <c r="H24" s="1" t="n"/>
       <c r="I24" s="1" t="n"/>
-      <c r="J24" s="29" t="inlineStr">
+      <c r="J24" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="K24" s="44" t="n">
+      <c r="K24" s="45" t="n">
         <v>1.2</v>
       </c>
       <c r="L24" s="1" t="n"/>
@@ -1866,35 +2091,36 @@
       <c r="Q24" s="1" t="n"/>
       <c r="R24" s="1" t="n"/>
       <c r="S24" s="1" t="n"/>
+      <c r="T24" s="1" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>Hausse tarifaire</t>
         </is>
       </c>
-      <c r="C25" s="42" t="n">
+      <c r="C25" s="43" t="n">
         <v>0.0029</v>
       </c>
-      <c r="D25" s="42" t="n">
+      <c r="D25" s="43" t="n">
         <v>0.035</v>
       </c>
-      <c r="E25" s="42" t="n">
+      <c r="E25" s="43" t="n">
         <v>0.02</v>
       </c>
-      <c r="F25" s="43" t="n">
+      <c r="F25" s="44" t="n">
         <v>0.035</v>
       </c>
       <c r="G25" s="1" t="n"/>
       <c r="H25" s="1" t="n"/>
       <c r="I25" s="1" t="n"/>
-      <c r="J25" s="29" t="inlineStr">
+      <c r="J25" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="K25" s="44" t="n">
+      <c r="K25" s="45" t="n">
         <v>1.15</v>
       </c>
       <c r="L25" s="1" t="n"/>
@@ -1905,35 +2131,36 @@
       <c r="Q25" s="1" t="n"/>
       <c r="R25" s="1" t="n"/>
       <c r="S25" s="1" t="n"/>
+      <c r="T25" s="1" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="29" t="inlineStr">
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Gain de conversion lead / candidature</t>
         </is>
       </c>
-      <c r="C26" s="42" t="n">
+      <c r="C26" s="43" t="n">
         <v>0.01</v>
       </c>
-      <c r="D26" s="42" t="n">
+      <c r="D26" s="43" t="n">
         <v>0.03</v>
       </c>
-      <c r="E26" s="42" t="n">
+      <c r="E26" s="43" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F26" s="43" t="n">
+      <c r="F26" s="44" t="n">
         <v>0.03</v>
       </c>
       <c r="G26" s="1" t="n"/>
       <c r="H26" s="1" t="n"/>
       <c r="I26" s="1" t="n"/>
-      <c r="J26" s="29" t="inlineStr">
+      <c r="J26" s="30" t="inlineStr">
         <is>
           <t>Ipac Bachelor Factory</t>
         </is>
       </c>
-      <c r="K26" s="44" t="n">
+      <c r="K26" s="45" t="n">
         <v>0.95</v>
       </c>
       <c r="L26" s="1" t="n"/>
@@ -1944,35 +2171,36 @@
       <c r="Q26" s="1" t="n"/>
       <c r="R26" s="1" t="n"/>
       <c r="S26" s="1" t="n"/>
+      <c r="T26" s="1" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>Gain de conversion admis / inscrit</t>
         </is>
       </c>
-      <c r="C27" s="42" t="n">
+      <c r="C27" s="43" t="n">
         <v>0.01</v>
       </c>
-      <c r="D27" s="42" t="n">
+      <c r="D27" s="43" t="n">
         <v>0.025</v>
       </c>
-      <c r="E27" s="42" t="n">
+      <c r="E27" s="43" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F27" s="43" t="n">
+      <c r="F27" s="44" t="n">
         <v>0.025</v>
       </c>
       <c r="G27" s="1" t="n"/>
       <c r="H27" s="1" t="n"/>
       <c r="I27" s="1" t="n"/>
-      <c r="J27" s="29" t="inlineStr">
+      <c r="J27" s="30" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="K27" s="44" t="n">
+      <c r="K27" s="45" t="n">
         <v>0.9</v>
       </c>
       <c r="L27" s="1" t="n"/>
@@ -1983,35 +2211,36 @@
       <c r="Q27" s="1" t="n"/>
       <c r="R27" s="1" t="n"/>
       <c r="S27" s="1" t="n"/>
+      <c r="T27" s="1" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="29" t="inlineStr">
+      <c r="B28" s="30" t="inlineStr">
         <is>
           <t>Amélioration du taux de passage</t>
         </is>
       </c>
-      <c r="C28" s="42" t="n">
+      <c r="C28" s="43" t="n">
         <v>0.005</v>
       </c>
-      <c r="D28" s="42" t="n">
+      <c r="D28" s="43" t="n">
         <v>0.015</v>
       </c>
-      <c r="E28" s="42" t="n">
+      <c r="E28" s="43" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F28" s="43" t="n">
+      <c r="F28" s="44" t="n">
         <v>0.015</v>
       </c>
       <c r="G28" s="1" t="n"/>
       <c r="H28" s="1" t="n"/>
       <c r="I28" s="1" t="n"/>
-      <c r="J28" s="29" t="inlineStr">
+      <c r="J28" s="30" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="K28" s="44" t="n">
+      <c r="K28" s="45" t="n">
         <v>1.05</v>
       </c>
       <c r="L28" s="1" t="n"/>
@@ -2022,6 +2251,7 @@
       <c r="Q28" s="1" t="n"/>
       <c r="R28" s="1" t="n"/>
       <c r="S28" s="1" t="n"/>
+      <c r="T28" s="1" t="n"/>
     </row>
     <row r="29" ht="6" customHeight="1">
       <c r="A29" s="1" t="n"/>
@@ -2043,6 +2273,7 @@
       <c r="Q29" s="1" t="n"/>
       <c r="R29" s="1" t="n"/>
       <c r="S29" s="1" t="n"/>
+      <c r="T29" s="1" t="n"/>
     </row>
     <row r="30" ht="6" customHeight="1">
       <c r="A30" s="1" t="n"/>
@@ -2064,6 +2295,7 @@
       <c r="Q30" s="1" t="n"/>
       <c r="R30" s="1" t="n"/>
       <c r="S30" s="1" t="n"/>
+      <c r="T30" s="1" t="n"/>
     </row>
     <row r="31" ht="6" customHeight="1">
       <c r="A31" s="1" t="n"/>
@@ -2085,18 +2317,19 @@
       <c r="Q31" s="1" t="n"/>
       <c r="R31" s="1" t="n"/>
       <c r="S31" s="1" t="n"/>
+      <c r="T31" s="1" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="39" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>Coûts</t>
         </is>
       </c>
-      <c r="C32" s="40" t="n"/>
-      <c r="D32" s="40" t="n"/>
-      <c r="E32" s="40" t="n"/>
-      <c r="F32" s="40" t="n"/>
+      <c r="C32" s="41" t="n"/>
+      <c r="D32" s="41" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="41" t="n"/>
       <c r="G32" s="1" t="n"/>
       <c r="H32" s="1" t="n"/>
       <c r="I32" s="1" t="n"/>
@@ -2110,6 +2343,7 @@
       <c r="Q32" s="1" t="n"/>
       <c r="R32" s="1" t="n"/>
       <c r="S32" s="1" t="n"/>
+      <c r="T32" s="1" t="n"/>
     </row>
     <row r="33" ht="6" customHeight="1">
       <c r="A33" s="1" t="n"/>
@@ -2131,24 +2365,25 @@
       <c r="Q33" s="1" t="n"/>
       <c r="R33" s="1" t="n"/>
       <c r="S33" s="1" t="n"/>
+      <c r="T33" s="1" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="n"/>
-      <c r="B34" s="29" t="inlineStr">
+      <c r="B34" s="30" t="inlineStr">
         <is>
           <t>Inflation des charges externes</t>
         </is>
       </c>
-      <c r="C34" s="42" t="n">
+      <c r="C34" s="43" t="n">
         <v>0.02</v>
       </c>
-      <c r="D34" s="42" t="n">
+      <c r="D34" s="43" t="n">
         <v>0.015</v>
       </c>
-      <c r="E34" s="42" t="n">
+      <c r="E34" s="43" t="n">
         <v>0.03</v>
       </c>
-      <c r="F34" s="43" t="n">
+      <c r="F34" s="44" t="n">
         <v>0.015</v>
       </c>
       <c r="G34" s="1" t="n"/>
@@ -2164,24 +2399,25 @@
       <c r="Q34" s="1" t="n"/>
       <c r="R34" s="1" t="n"/>
       <c r="S34" s="1" t="n"/>
+      <c r="T34" s="1" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="29" t="inlineStr">
+      <c r="B35" s="30" t="inlineStr">
         <is>
           <t>Politique salariale</t>
         </is>
       </c>
-      <c r="C35" s="42" t="n">
+      <c r="C35" s="43" t="n">
         <v>0.025</v>
       </c>
-      <c r="D35" s="42" t="n">
+      <c r="D35" s="43" t="n">
         <v>0.02</v>
       </c>
-      <c r="E35" s="42" t="n">
+      <c r="E35" s="43" t="n">
         <v>0.03</v>
       </c>
-      <c r="F35" s="43" t="n">
+      <c r="F35" s="44" t="n">
         <v>0.02</v>
       </c>
       <c r="G35" s="1" t="n"/>
@@ -2197,24 +2433,25 @@
       <c r="Q35" s="1" t="n"/>
       <c r="R35" s="1" t="n"/>
       <c r="S35" s="1" t="n"/>
+      <c r="T35" s="1" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="29" t="inlineStr">
+      <c r="B36" s="30" t="inlineStr">
         <is>
           <t>Variation des effectifs permanents</t>
         </is>
       </c>
-      <c r="C36" s="42" t="n">
+      <c r="C36" s="43" t="n">
         <v>0.04</v>
       </c>
-      <c r="D36" s="42" t="n">
+      <c r="D36" s="43" t="n">
         <v>0.03</v>
       </c>
-      <c r="E36" s="42" t="n">
+      <c r="E36" s="43" t="n">
         <v>0.05</v>
       </c>
-      <c r="F36" s="43" t="n">
+      <c r="F36" s="44" t="n">
         <v>0.03</v>
       </c>
       <c r="G36" s="1" t="n"/>
@@ -2230,26 +2467,27 @@
       <c r="Q36" s="1" t="n"/>
       <c r="R36" s="1" t="n"/>
       <c r="S36" s="1" t="n"/>
+      <c r="T36" s="1" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="29" t="inlineStr">
+      <c r="B37" s="30" t="inlineStr">
         <is>
           <t>Effort de productivité</t>
         </is>
       </c>
-      <c r="C37" s="42" t="n">
+      <c r="C37" s="43" t="n">
         <v>0.0185</v>
       </c>
-      <c r="D37" s="42" t="n">
+      <c r="D37" s="43" t="n">
         <v>0.03</v>
       </c>
-      <c r="E37" s="45" t="inlineStr">
+      <c r="E37" s="46" t="inlineStr">
         <is>
           <t>n.d.</t>
         </is>
       </c>
-      <c r="F37" s="43" t="n">
+      <c r="F37" s="44" t="n">
         <v>0.03</v>
       </c>
       <c r="G37" s="1" t="n"/>
@@ -2265,26 +2503,27 @@
       <c r="Q37" s="1" t="n"/>
       <c r="R37" s="1" t="n"/>
       <c r="S37" s="1" t="n"/>
+      <c r="T37" s="1" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="29" t="inlineStr">
+      <c r="B38" s="30" t="inlineStr">
         <is>
           <t>Variation des coûts de structure</t>
         </is>
       </c>
-      <c r="C38" s="45" t="inlineStr">
+      <c r="C38" s="46" t="inlineStr">
         <is>
           <t>n.d.</t>
         </is>
       </c>
-      <c r="D38" s="42" t="n">
+      <c r="D38" s="43" t="n">
         <v>-0.03</v>
       </c>
-      <c r="E38" s="42" t="n">
+      <c r="E38" s="43" t="n">
         <v>0.04</v>
       </c>
-      <c r="F38" s="43" t="n">
+      <c r="F38" s="44" t="n">
         <v>-0.03</v>
       </c>
       <c r="G38" s="1" t="n"/>
@@ -2300,6 +2539,7 @@
       <c r="Q38" s="1" t="n"/>
       <c r="R38" s="1" t="n"/>
       <c r="S38" s="1" t="n"/>
+      <c r="T38" s="1" t="n"/>
     </row>
     <row r="39" ht="6" customHeight="1">
       <c r="A39" s="1" t="n"/>
@@ -2321,18 +2561,19 @@
       <c r="Q39" s="1" t="n"/>
       <c r="R39" s="1" t="n"/>
       <c r="S39" s="1" t="n"/>
+      <c r="T39" s="1" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="39" t="inlineStr">
+      <c r="B40" s="40" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="C40" s="40" t="n"/>
-      <c r="D40" s="40" t="n"/>
-      <c r="E40" s="40" t="n"/>
-      <c r="F40" s="40" t="n"/>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="41" t="n"/>
       <c r="G40" s="1" t="n"/>
       <c r="H40" s="1" t="n"/>
       <c r="I40" s="1" t="n"/>
@@ -2346,6 +2587,7 @@
       <c r="Q40" s="1" t="n"/>
       <c r="R40" s="1" t="n"/>
       <c r="S40" s="1" t="n"/>
+      <c r="T40" s="1" t="n"/>
     </row>
     <row r="41" ht="6" customHeight="1">
       <c r="A41" s="1" t="n"/>
@@ -2367,24 +2609,25 @@
       <c r="Q41" s="1" t="n"/>
       <c r="R41" s="1" t="n"/>
       <c r="S41" s="1" t="n"/>
+      <c r="T41" s="1" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="n"/>
-      <c r="B42" s="29" t="inlineStr">
+      <c r="B42" s="30" t="inlineStr">
         <is>
           <t>Frais de dossier par nouvel inscrit</t>
         </is>
       </c>
-      <c r="C42" s="46" t="n">
+      <c r="C42" s="47" t="n">
         <v>90</v>
       </c>
-      <c r="D42" s="46" t="n">
+      <c r="D42" s="47" t="n">
         <v>90</v>
       </c>
-      <c r="E42" s="46" t="n">
+      <c r="E42" s="47" t="n">
         <v>90</v>
       </c>
-      <c r="F42" s="47" t="n">
+      <c r="F42" s="48" t="n">
         <v>90</v>
       </c>
       <c r="G42" s="1" t="n"/>
@@ -2400,6 +2643,7 @@
       <c r="Q42" s="1" t="n"/>
       <c r="R42" s="1" t="n"/>
       <c r="S42" s="1" t="n"/>
+      <c r="T42" s="1" t="n"/>
     </row>
     <row r="43" ht="12" customHeight="1">
       <c r="A43" s="1" t="n"/>
@@ -2421,10 +2665,11 @@
       <c r="Q43" s="1" t="n"/>
       <c r="R43" s="1" t="n"/>
       <c r="S43" s="1" t="n"/>
+      <c r="T43" s="1" t="n"/>
     </row>
     <row r="44" ht="12" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="48" t="inlineStr">
+      <c r="B44" s="49" t="inlineStr">
         <is>
           <t>Source : Tagetik TGK_MSSQL_07, cube d'hypothèses, versions V01 / V02 / V03.</t>
         </is>
@@ -2446,6 +2691,7 @@
       <c r="Q44" s="1" t="n"/>
       <c r="R44" s="1" t="n"/>
       <c r="S44" s="1" t="n"/>
+      <c r="T44" s="1" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n"/>
@@ -2467,6 +2713,7 @@
       <c r="Q45" s="1" t="n"/>
       <c r="R45" s="1" t="n"/>
       <c r="S45" s="1" t="n"/>
+      <c r="T45" s="1" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n"/>
@@ -2488,6 +2735,7 @@
       <c r="Q46" s="1" t="n"/>
       <c r="R46" s="1" t="n"/>
       <c r="S46" s="1" t="n"/>
+      <c r="T46" s="1" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2747,36 +2995,36 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>EBITDA après siège</t>
         </is>
       </c>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Marge EBITDA</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Effectif moyen</t>
         </is>
       </c>
-      <c r="H9" s="15" t="n"/>
-      <c r="I9" s="14" t="inlineStr">
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>Croissance CA</t>
         </is>
       </c>
-      <c r="J9" s="15" t="n"/>
-      <c r="K9" s="16" t="n"/>
+      <c r="J9" s="16" t="n"/>
+      <c r="K9" s="17" t="n"/>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
       <c r="N9" s="1" t="n"/>
@@ -2792,26 +3040,26 @@
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="18" t="n">
         <v>24231703.55</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="19" t="n">
         <v>4111503.64</v>
       </c>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="49" t="n">
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="50" t="n">
         <v>0.1697</v>
       </c>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="50" t="n">
+      <c r="F10" s="20" t="n"/>
+      <c r="G10" s="51" t="n">
         <v>3253.62</v>
       </c>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="49" t="n">
+      <c r="H10" s="20" t="n"/>
+      <c r="I10" s="50" t="n">
         <v>0.049</v>
       </c>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="20" t="n"/>
+      <c r="J10" s="20" t="n"/>
+      <c r="K10" s="21" t="n"/>
       <c r="L10" s="1" t="n"/>
       <c r="M10" s="1" t="n"/>
       <c r="N10" s="1" t="n"/>
@@ -2827,36 +3075,36 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>2026 : 23 098 985 €</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>2026 : 3 845 790 €</t>
         </is>
       </c>
-      <c r="D11" s="23" t="n"/>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="23" t="inlineStr">
         <is>
           <t>2026 : 16,6 %</t>
         </is>
       </c>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="22" t="inlineStr">
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>2026 : 3 114</t>
         </is>
       </c>
-      <c r="H11" s="23" t="n"/>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="23" t="inlineStr">
         <is>
           <t>vs réel 2026</t>
         </is>
       </c>
-      <c r="J11" s="23" t="n"/>
-      <c r="K11" s="24" t="n"/>
+      <c r="J11" s="24" t="n"/>
+      <c r="K11" s="25" t="n"/>
       <c r="L11" s="1" t="n"/>
       <c r="M11" s="1" t="n"/>
       <c r="N11" s="1" t="n"/>
@@ -2972,21 +3220,21 @@
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>CAPACITÉ PAR CAMPUS</t>
         </is>
       </c>
-      <c r="C16" s="26" t="n"/>
-      <c r="D16" s="26" t="n"/>
-      <c r="E16" s="26" t="n"/>
-      <c r="F16" s="26" t="n"/>
-      <c r="G16" s="26" t="n"/>
-      <c r="H16" s="26" t="n"/>
-      <c r="I16" s="26" t="n"/>
-      <c r="J16" s="26" t="n"/>
-      <c r="K16" s="26" t="n"/>
-      <c r="L16" s="26" t="n"/>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="27" t="n"/>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="27" t="n"/>
       <c r="M16" s="1" t="n"/>
       <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
@@ -3025,58 +3273,58 @@
       <c r="W17" s="1" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="51" t="inlineStr"/>
-      <c r="B18" s="52" t="inlineStr">
+      <c r="A18" s="52" t="inlineStr"/>
+      <c r="B18" s="53" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="C18" s="52" t="inlineStr">
+      <c r="C18" s="53" t="inlineStr">
         <is>
           <t>Ville</t>
         </is>
       </c>
-      <c r="D18" s="53" t="inlineStr">
+      <c r="D18" s="54" t="inlineStr">
         <is>
           <t>CAC marginal</t>
         </is>
       </c>
-      <c r="E18" s="53" t="inlineStr">
+      <c r="E18" s="54" t="inlineStr">
         <is>
           <t>Croissance leads</t>
         </is>
       </c>
-      <c r="F18" s="53" t="inlineStr">
+      <c r="F18" s="54" t="inlineStr">
         <is>
           <t>Intensité marketing</t>
         </is>
       </c>
-      <c r="G18" s="51" t="inlineStr">
+      <c r="G18" s="52" t="inlineStr">
         <is>
           <t>Cap effectif</t>
         </is>
       </c>
-      <c r="H18" s="51" t="inlineStr">
+      <c r="H18" s="52" t="inlineStr">
         <is>
           <t>Cap momentum</t>
         </is>
       </c>
-      <c r="I18" s="51" t="inlineStr">
+      <c r="I18" s="52" t="inlineStr">
         <is>
           <t>Cap potentiel</t>
         </is>
       </c>
-      <c r="J18" s="54" t="inlineStr">
+      <c r="J18" s="55" t="inlineStr">
         <is>
           <t>Cap retenu</t>
         </is>
       </c>
-      <c r="K18" s="53" t="inlineStr">
+      <c r="K18" s="54" t="inlineStr">
         <is>
           <t>Budget acquisition</t>
         </is>
       </c>
-      <c r="L18" s="52" t="inlineStr">
+      <c r="L18" s="53" t="inlineStr">
         <is>
           <t>Code campus</t>
         </is>
@@ -3094,42 +3342,42 @@
       <c r="W18" s="1" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="55" t="inlineStr"/>
-      <c r="B19" s="29" t="inlineStr">
+      <c r="A19" s="56" t="inlineStr"/>
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C19" s="56" t="inlineStr">
+      <c r="C19" s="57" t="inlineStr">
         <is>
           <t>Montpellier</t>
         </is>
       </c>
-      <c r="D19" s="30" t="n">
+      <c r="D19" s="31" t="n">
         <v>1033.98</v>
       </c>
-      <c r="E19" s="31" t="n">
+      <c r="E19" s="32" t="n">
         <v>0.1448</v>
       </c>
-      <c r="F19" s="31" t="n">
+      <c r="F19" s="32" t="n">
         <v>0.0194</v>
       </c>
-      <c r="G19" s="44" t="n">
+      <c r="G19" s="45" t="n">
         <v>1.1626</v>
       </c>
-      <c r="H19" s="44" t="n">
+      <c r="H19" s="45" t="n">
         <v>1.3855</v>
       </c>
-      <c r="I19" s="44" t="n">
+      <c r="I19" s="45" t="n">
         <v>0.9443</v>
       </c>
-      <c r="J19" s="57" t="n">
+      <c r="J19" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K19" s="30" t="n">
+      <c r="K19" s="31" t="n">
         <v>15178</v>
       </c>
-      <c r="L19" s="58" t="inlineStr">
+      <c r="L19" s="59" t="inlineStr">
         <is>
           <t>IPAC_MTP</t>
         </is>
@@ -3147,42 +3395,42 @@
       <c r="W19" s="1" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="55" t="inlineStr"/>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="A20" s="56" t="inlineStr"/>
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C20" s="56" t="inlineStr">
+      <c r="C20" s="57" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D20" s="30" t="n">
+      <c r="D20" s="31" t="n">
         <v>1216.29</v>
       </c>
-      <c r="E20" s="31" t="n">
+      <c r="E20" s="32" t="n">
         <v>0.1379</v>
       </c>
-      <c r="F20" s="31" t="n">
+      <c r="F20" s="32" t="n">
         <v>0.0213</v>
       </c>
-      <c r="G20" s="44" t="n">
+      <c r="G20" s="45" t="n">
         <v>0.9883</v>
       </c>
-      <c r="H20" s="44" t="n">
+      <c r="H20" s="45" t="n">
         <v>1.3195</v>
       </c>
-      <c r="I20" s="44" t="n">
+      <c r="I20" s="45" t="n">
         <v>0.8591</v>
       </c>
-      <c r="J20" s="57" t="n">
+      <c r="J20" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K20" s="30" t="n">
+      <c r="K20" s="31" t="n">
         <v>21760</v>
       </c>
-      <c r="L20" s="58" t="inlineStr">
+      <c r="L20" s="59" t="inlineStr">
         <is>
           <t>IPAC_NAN</t>
         </is>
@@ -3200,42 +3448,42 @@
       <c r="W20" s="1" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="55" t="inlineStr"/>
-      <c r="B21" s="29" t="inlineStr">
+      <c r="A21" s="56" t="inlineStr"/>
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C21" s="56" t="inlineStr">
+      <c r="C21" s="57" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="D21" s="30" t="n">
+      <c r="D21" s="31" t="n">
         <v>1040.56</v>
       </c>
-      <c r="E21" s="31" t="n">
+      <c r="E21" s="32" t="n">
         <v>0.1448</v>
       </c>
-      <c r="F21" s="31" t="n">
+      <c r="F21" s="32" t="n">
         <v>0.0191</v>
       </c>
-      <c r="G21" s="44" t="n">
+      <c r="G21" s="45" t="n">
         <v>1.1553</v>
       </c>
-      <c r="H21" s="44" t="n">
+      <c r="H21" s="45" t="n">
         <v>1.3855</v>
       </c>
-      <c r="I21" s="44" t="n">
+      <c r="I21" s="45" t="n">
         <v>0.9598</v>
       </c>
-      <c r="J21" s="57" t="n">
+      <c r="J21" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K21" s="30" t="n">
+      <c r="K21" s="31" t="n">
         <v>14933</v>
       </c>
-      <c r="L21" s="58" t="inlineStr">
+      <c r="L21" s="59" t="inlineStr">
         <is>
           <t>IPAC_REN</t>
         </is>
@@ -3253,42 +3501,42 @@
       <c r="W21" s="1" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="55" t="inlineStr"/>
-      <c r="B22" s="29" t="inlineStr">
+      <c r="A22" s="56" t="inlineStr"/>
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C22" s="56" t="inlineStr">
+      <c r="C22" s="57" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="D22" s="30" t="n">
+      <c r="D22" s="31" t="n">
         <v>978.58</v>
       </c>
-      <c r="E22" s="31" t="n">
+      <c r="E22" s="32" t="n">
         <v>0.0815</v>
       </c>
-      <c r="F22" s="31" t="n">
+      <c r="F22" s="32" t="n">
         <v>0.0144</v>
       </c>
-      <c r="G22" s="44" t="n">
+      <c r="G22" s="45" t="n">
         <v>1.2284</v>
       </c>
-      <c r="H22" s="44" t="n">
+      <c r="H22" s="45" t="n">
         <v>0.7804</v>
       </c>
-      <c r="I22" s="44" t="n">
+      <c r="I22" s="45" t="n">
         <v>1.2767</v>
       </c>
-      <c r="J22" s="57" t="n">
+      <c r="J22" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="30" t="n">
+      <c r="K22" s="31" t="n">
         <v>25220</v>
       </c>
-      <c r="L22" s="58" t="inlineStr">
+      <c r="L22" s="59" t="inlineStr">
         <is>
           <t>ISCOM_LIL</t>
         </is>
@@ -3306,42 +3554,42 @@
       <c r="W22" s="1" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="55" t="inlineStr"/>
-      <c r="B23" s="29" t="inlineStr">
+      <c r="A23" s="56" t="inlineStr"/>
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C23" s="56" t="inlineStr">
+      <c r="C23" s="57" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D23" s="30" t="n">
+      <c r="D23" s="31" t="n">
         <v>1540.33</v>
       </c>
-      <c r="E23" s="31" t="n">
+      <c r="E23" s="32" t="n">
         <v>0.07770000000000001</v>
       </c>
-      <c r="F23" s="31" t="n">
+      <c r="F23" s="32" t="n">
         <v>0.0209</v>
       </c>
-      <c r="G23" s="44" t="n">
+      <c r="G23" s="45" t="n">
         <v>0.7804</v>
       </c>
-      <c r="H23" s="44" t="n">
+      <c r="H23" s="45" t="n">
         <v>0.744</v>
       </c>
-      <c r="I23" s="44" t="n">
+      <c r="I23" s="45" t="n">
         <v>0.8773</v>
       </c>
-      <c r="J23" s="57" t="n">
+      <c r="J23" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K23" s="30" t="n">
+      <c r="K23" s="31" t="n">
         <v>60800</v>
       </c>
-      <c r="L23" s="58" t="inlineStr">
+      <c r="L23" s="59" t="inlineStr">
         <is>
           <t>ISCOM_PAR</t>
         </is>
@@ -3359,42 +3607,42 @@
       <c r="W23" s="1" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="55" t="inlineStr"/>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="A24" s="56" t="inlineStr"/>
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C24" s="56" t="inlineStr">
+      <c r="C24" s="57" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="D24" s="30" t="n">
+      <c r="D24" s="31" t="n">
         <v>919.03</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="32" t="n">
         <v>0.08210000000000001</v>
       </c>
-      <c r="F24" s="31" t="n">
+      <c r="F24" s="32" t="n">
         <v>0.0136</v>
       </c>
-      <c r="G24" s="44" t="n">
+      <c r="G24" s="45" t="n">
         <v>1.308</v>
       </c>
-      <c r="H24" s="44" t="n">
+      <c r="H24" s="45" t="n">
         <v>0.7858000000000001</v>
       </c>
-      <c r="I24" s="44" t="n">
+      <c r="I24" s="45" t="n">
         <v>1.3518</v>
       </c>
-      <c r="J24" s="57" t="n">
+      <c r="J24" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K24" s="30" t="n">
+      <c r="K24" s="31" t="n">
         <v>22083</v>
       </c>
-      <c r="L24" s="58" t="inlineStr">
+      <c r="L24" s="59" t="inlineStr">
         <is>
           <t>ISCOM_TLS</t>
         </is>
@@ -3412,42 +3660,42 @@
       <c r="W24" s="1" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="55" t="inlineStr"/>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="A25" s="56" t="inlineStr"/>
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C25" s="56" t="inlineStr">
+      <c r="C25" s="57" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D25" s="30" t="n">
+      <c r="D25" s="31" t="n">
         <v>889.59</v>
       </c>
-      <c r="E25" s="31" t="n">
+      <c r="E25" s="32" t="n">
         <v>0.1261</v>
       </c>
-      <c r="F25" s="31" t="n">
+      <c r="F25" s="32" t="n">
         <v>0.0141</v>
       </c>
-      <c r="G25" s="44" t="n">
+      <c r="G25" s="45" t="n">
         <v>1.3513</v>
       </c>
-      <c r="H25" s="44" t="n">
+      <c r="H25" s="45" t="n">
         <v>1.2067</v>
       </c>
-      <c r="I25" s="44" t="n">
+      <c r="I25" s="45" t="n">
         <v>1.3049</v>
       </c>
-      <c r="J25" s="57" t="n">
+      <c r="J25" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="30" t="n">
+      <c r="K25" s="31" t="n">
         <v>24923</v>
       </c>
-      <c r="L25" s="58" t="inlineStr">
+      <c r="L25" s="59" t="inlineStr">
         <is>
           <t>MBWAY_BOR</t>
         </is>
@@ -3465,42 +3713,42 @@
       <c r="W25" s="1" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="55" t="inlineStr"/>
-      <c r="B26" s="29" t="inlineStr">
+      <c r="A26" s="56" t="inlineStr"/>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C26" s="56" t="inlineStr">
+      <c r="C26" s="57" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D26" s="30" t="n">
+      <c r="D26" s="31" t="n">
         <v>1101.6</v>
       </c>
-      <c r="E26" s="31" t="n">
+      <c r="E26" s="32" t="n">
         <v>0.1189</v>
       </c>
-      <c r="F26" s="31" t="n">
+      <c r="F26" s="32" t="n">
         <v>0.0167</v>
       </c>
-      <c r="G26" s="44" t="n">
+      <c r="G26" s="45" t="n">
         <v>1.0912</v>
       </c>
-      <c r="H26" s="44" t="n">
+      <c r="H26" s="45" t="n">
         <v>1.1376</v>
       </c>
-      <c r="I26" s="44" t="n">
+      <c r="I26" s="45" t="n">
         <v>1.0957</v>
       </c>
-      <c r="J26" s="57" t="n">
+      <c r="J26" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K26" s="30" t="n">
+      <c r="K26" s="31" t="n">
         <v>41783</v>
       </c>
-      <c r="L26" s="58" t="inlineStr">
+      <c r="L26" s="59" t="inlineStr">
         <is>
           <t>MBWAY_LYO</t>
         </is>
@@ -3518,42 +3766,42 @@
       <c r="W26" s="1" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="55" t="inlineStr"/>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="A27" s="56" t="inlineStr"/>
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C27" s="56" t="inlineStr">
+      <c r="C27" s="57" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D27" s="30" t="n">
+      <c r="D27" s="31" t="n">
         <v>963.58</v>
       </c>
-      <c r="E27" s="31" t="n">
+      <c r="E27" s="32" t="n">
         <v>0.1238</v>
       </c>
-      <c r="F27" s="31" t="n">
+      <c r="F27" s="32" t="n">
         <v>0.0146</v>
       </c>
-      <c r="G27" s="44" t="n">
+      <c r="G27" s="45" t="n">
         <v>1.2476</v>
       </c>
-      <c r="H27" s="44" t="n">
+      <c r="H27" s="45" t="n">
         <v>1.1847</v>
       </c>
-      <c r="I27" s="44" t="n">
+      <c r="I27" s="45" t="n">
         <v>1.2551</v>
       </c>
-      <c r="J27" s="57" t="n">
+      <c r="J27" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K27" s="30" t="n">
+      <c r="K27" s="31" t="n">
         <v>31533</v>
       </c>
-      <c r="L27" s="58" t="inlineStr">
+      <c r="L27" s="59" t="inlineStr">
         <is>
           <t>MBWAY_NAN</t>
         </is>
@@ -3571,42 +3819,42 @@
       <c r="W27" s="1" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="55" t="inlineStr"/>
-      <c r="B28" s="29" t="inlineStr">
+      <c r="A28" s="56" t="inlineStr"/>
+      <c r="B28" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C28" s="56" t="inlineStr">
+      <c r="C28" s="57" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D28" s="30" t="n">
+      <c r="D28" s="31" t="n">
         <v>1475.02</v>
       </c>
-      <c r="E28" s="31" t="n">
+      <c r="E28" s="32" t="n">
         <v>0.1107</v>
       </c>
-      <c r="F28" s="31" t="n">
+      <c r="F28" s="32" t="n">
         <v>0.0218</v>
       </c>
-      <c r="G28" s="44" t="n">
+      <c r="G28" s="45" t="n">
         <v>0.8149999999999999</v>
       </c>
-      <c r="H28" s="44" t="n">
+      <c r="H28" s="45" t="n">
         <v>1.0597</v>
       </c>
-      <c r="I28" s="44" t="n">
+      <c r="I28" s="45" t="n">
         <v>0.8428</v>
       </c>
-      <c r="J28" s="57" t="n">
+      <c r="J28" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K28" s="30" t="n">
+      <c r="K28" s="31" t="n">
         <v>68291</v>
       </c>
-      <c r="L28" s="58" t="inlineStr">
+      <c r="L28" s="59" t="inlineStr">
         <is>
           <t>MBWAY_PAR</t>
         </is>
@@ -3624,42 +3872,42 @@
       <c r="W28" s="1" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="55" t="inlineStr"/>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="A29" s="56" t="inlineStr"/>
+      <c r="B29" s="30" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C29" s="56" t="inlineStr">
+      <c r="C29" s="57" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D29" s="30" t="n">
+      <c r="D29" s="31" t="n">
         <v>1368.09</v>
       </c>
-      <c r="E29" s="31" t="n">
+      <c r="E29" s="32" t="n">
         <v>0.08749999999999999</v>
       </c>
-      <c r="F29" s="31" t="n">
+      <c r="F29" s="32" t="n">
         <v>0.0194</v>
       </c>
-      <c r="G29" s="44" t="n">
+      <c r="G29" s="45" t="n">
         <v>0.8787</v>
       </c>
-      <c r="H29" s="44" t="n">
+      <c r="H29" s="45" t="n">
         <v>0.8377</v>
       </c>
-      <c r="I29" s="44" t="n">
+      <c r="I29" s="45" t="n">
         <v>0.9454</v>
       </c>
-      <c r="J29" s="57" t="n">
+      <c r="J29" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K29" s="30" t="n">
+      <c r="K29" s="31" t="n">
         <v>21968</v>
       </c>
-      <c r="L29" s="58" t="inlineStr">
+      <c r="L29" s="59" t="inlineStr">
         <is>
           <t>PIGIER_BOR</t>
         </is>
@@ -3677,42 +3925,42 @@
       <c r="W29" s="1" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="55" t="inlineStr"/>
-      <c r="B30" s="29" t="inlineStr">
+      <c r="A30" s="56" t="inlineStr"/>
+      <c r="B30" s="30" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C30" s="56" t="inlineStr">
+      <c r="C30" s="57" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D30" s="30" t="n">
+      <c r="D30" s="31" t="n">
         <v>1704.98</v>
       </c>
-      <c r="E30" s="31" t="n">
+      <c r="E30" s="32" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="F30" s="31" t="n">
+      <c r="F30" s="32" t="n">
         <v>0.0233</v>
       </c>
-      <c r="G30" s="44" t="n">
+      <c r="G30" s="45" t="n">
         <v>0.7050999999999999</v>
       </c>
-      <c r="H30" s="44" t="n">
+      <c r="H30" s="45" t="n">
         <v>0.8135</v>
       </c>
-      <c r="I30" s="44" t="n">
+      <c r="I30" s="45" t="n">
         <v>0.7883</v>
       </c>
-      <c r="J30" s="57" t="n">
+      <c r="J30" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K30" s="30" t="n">
+      <c r="K30" s="31" t="n">
         <v>36612</v>
       </c>
-      <c r="L30" s="58" t="inlineStr">
+      <c r="L30" s="59" t="inlineStr">
         <is>
           <t>PIGIER_LYO</t>
         </is>
@@ -3730,42 +3978,42 @@
       <c r="W30" s="1" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="55" t="inlineStr"/>
-      <c r="B31" s="29" t="inlineStr">
+      <c r="A31" s="56" t="inlineStr"/>
+      <c r="B31" s="30" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C31" s="56" t="inlineStr">
+      <c r="C31" s="57" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D31" s="30" t="n">
+      <c r="D31" s="31" t="n">
         <v>1624.68</v>
       </c>
-      <c r="E31" s="31" t="n">
+      <c r="E31" s="32" t="n">
         <v>0.0726</v>
       </c>
-      <c r="F31" s="31" t="n">
+      <c r="F31" s="32" t="n">
         <v>0.0218</v>
       </c>
-      <c r="G31" s="44" t="n">
+      <c r="G31" s="45" t="n">
         <v>0.7399</v>
       </c>
-      <c r="H31" s="44" t="n">
+      <c r="H31" s="45" t="n">
         <v>0.6943</v>
       </c>
-      <c r="I31" s="44" t="n">
+      <c r="I31" s="45" t="n">
         <v>0.8401</v>
       </c>
-      <c r="J31" s="57" t="n">
+      <c r="J31" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K31" s="30" t="n">
+      <c r="K31" s="31" t="n">
         <v>18850</v>
       </c>
-      <c r="L31" s="58" t="inlineStr">
+      <c r="L31" s="59" t="inlineStr">
         <is>
           <t>TUNON_LYO</t>
         </is>
@@ -3783,42 +4031,42 @@
       <c r="W31" s="1" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="55" t="inlineStr"/>
-      <c r="B32" s="29" t="inlineStr">
+      <c r="A32" s="56" t="inlineStr"/>
+      <c r="B32" s="30" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C32" s="56" t="inlineStr">
+      <c r="C32" s="57" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D32" s="30" t="n">
+      <c r="D32" s="31" t="n">
         <v>2192.89</v>
       </c>
-      <c r="E32" s="31" t="n">
+      <c r="E32" s="32" t="n">
         <v>0.06950000000000001</v>
       </c>
-      <c r="F32" s="31" t="n">
+      <c r="F32" s="32" t="n">
         <v>0.0278</v>
       </c>
-      <c r="G32" s="44" t="n">
+      <c r="G32" s="45" t="n">
         <v>0.5482</v>
       </c>
-      <c r="H32" s="44" t="n">
+      <c r="H32" s="45" t="n">
         <v>0.6653</v>
       </c>
-      <c r="I32" s="44" t="n">
+      <c r="I32" s="45" t="n">
         <v>0.6586</v>
       </c>
-      <c r="J32" s="57" t="n">
+      <c r="J32" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="K32" s="30" t="n">
+      <c r="K32" s="31" t="n">
         <v>30240</v>
       </c>
-      <c r="L32" s="58" t="inlineStr">
+      <c r="L32" s="59" t="inlineStr">
         <is>
           <t>TUNON_PAR</t>
         </is>
@@ -3912,21 +4160,21 @@
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>SYNTHÈSE PAR CAMPUS</t>
         </is>
       </c>
-      <c r="C36" s="26" t="n"/>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="26" t="n"/>
-      <c r="F36" s="26" t="n"/>
-      <c r="G36" s="26" t="n"/>
-      <c r="H36" s="26" t="n"/>
-      <c r="I36" s="26" t="n"/>
-      <c r="J36" s="26" t="n"/>
-      <c r="K36" s="26" t="n"/>
-      <c r="L36" s="26" t="n"/>
+      <c r="C36" s="27" t="n"/>
+      <c r="D36" s="27" t="n"/>
+      <c r="E36" s="27" t="n"/>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
+      <c r="H36" s="27" t="n"/>
+      <c r="I36" s="27" t="n"/>
+      <c r="J36" s="27" t="n"/>
+      <c r="K36" s="27" t="n"/>
+      <c r="L36" s="27" t="n"/>
       <c r="M36" s="1" t="n"/>
       <c r="N36" s="1" t="n"/>
       <c r="O36" s="1" t="n"/>
@@ -3965,58 +4213,58 @@
       <c r="W37" s="1" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="51" t="inlineStr"/>
-      <c r="B38" s="52" t="inlineStr">
+      <c r="A38" s="52" t="inlineStr"/>
+      <c r="B38" s="53" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="C38" s="52" t="inlineStr">
+      <c r="C38" s="53" t="inlineStr">
         <is>
           <t>Ville</t>
         </is>
       </c>
-      <c r="D38" s="53" t="inlineStr">
+      <c r="D38" s="54" t="inlineStr">
         <is>
           <t>Effectif</t>
         </is>
       </c>
-      <c r="E38" s="53" t="inlineStr">
+      <c r="E38" s="54" t="inlineStr">
         <is>
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="F38" s="53" t="inlineStr">
+      <c r="F38" s="54" t="inlineStr">
         <is>
           <t>Prix moyen</t>
         </is>
       </c>
-      <c r="G38" s="53" t="inlineStr">
+      <c r="G38" s="54" t="inlineStr">
         <is>
           <t>Part du CA</t>
         </is>
       </c>
-      <c r="H38" s="53" t="inlineStr">
+      <c r="H38" s="54" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="I38" s="51" t="inlineStr">
+      <c r="I38" s="52" t="inlineStr">
         <is>
           <t>Marge</t>
         </is>
       </c>
-      <c r="J38" s="53" t="inlineStr">
+      <c r="J38" s="54" t="inlineStr">
         <is>
           <t>EBITDA par étudiant</t>
         </is>
       </c>
-      <c r="K38" s="53" t="inlineStr">
+      <c r="K38" s="54" t="inlineStr">
         <is>
           <t>Budget acquisition</t>
         </is>
       </c>
-      <c r="L38" s="53" t="inlineStr">
+      <c r="L38" s="54" t="inlineStr">
         <is>
           <t>CAC marginal</t>
         </is>
@@ -4034,42 +4282,42 @@
       <c r="W38" s="1" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="55" t="inlineStr"/>
-      <c r="B39" s="29" t="inlineStr">
+      <c r="A39" s="56" t="inlineStr"/>
+      <c r="B39" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C39" s="56" t="inlineStr">
+      <c r="C39" s="57" t="inlineStr">
         <is>
           <t>Montpellier</t>
         </is>
       </c>
-      <c r="D39" s="59" t="n">
+      <c r="D39" s="60" t="n">
         <v>122.13</v>
       </c>
-      <c r="E39" s="30" t="n">
+      <c r="E39" s="31" t="n">
         <v>818445.73</v>
       </c>
-      <c r="F39" s="30" t="n">
+      <c r="F39" s="31" t="n">
         <v>6701.29</v>
       </c>
-      <c r="G39" s="31" t="n">
+      <c r="G39" s="32" t="n">
         <v>0.0338</v>
       </c>
-      <c r="H39" s="30" t="n">
+      <c r="H39" s="31" t="n">
         <v>254308.3</v>
       </c>
-      <c r="I39" s="60" t="n">
+      <c r="I39" s="61" t="n">
         <v>0.3107</v>
       </c>
-      <c r="J39" s="30" t="n">
+      <c r="J39" s="31" t="n">
         <v>2082.23</v>
       </c>
-      <c r="K39" s="30" t="n">
+      <c r="K39" s="31" t="n">
         <v>15178</v>
       </c>
-      <c r="L39" s="30" t="n">
+      <c r="L39" s="31" t="n">
         <v>1033.98</v>
       </c>
       <c r="M39" s="1" t="n"/>
@@ -4085,42 +4333,42 @@
       <c r="W39" s="1" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="55" t="inlineStr"/>
-      <c r="B40" s="29" t="inlineStr">
+      <c r="A40" s="56" t="inlineStr"/>
+      <c r="B40" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C40" s="56" t="inlineStr">
+      <c r="C40" s="57" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D40" s="59" t="n">
+      <c r="D40" s="60" t="n">
         <v>151.32</v>
       </c>
-      <c r="E40" s="30" t="n">
+      <c r="E40" s="31" t="n">
         <v>1067200.79</v>
       </c>
-      <c r="F40" s="30" t="n">
+      <c r="F40" s="31" t="n">
         <v>7052.49</v>
       </c>
-      <c r="G40" s="31" t="n">
+      <c r="G40" s="32" t="n">
         <v>0.044</v>
       </c>
-      <c r="H40" s="30" t="n">
+      <c r="H40" s="31" t="n">
         <v>331184.51</v>
       </c>
-      <c r="I40" s="60" t="n">
+      <c r="I40" s="61" t="n">
         <v>0.3103</v>
       </c>
-      <c r="J40" s="30" t="n">
+      <c r="J40" s="31" t="n">
         <v>2188.6</v>
       </c>
-      <c r="K40" s="30" t="n">
+      <c r="K40" s="31" t="n">
         <v>21760</v>
       </c>
-      <c r="L40" s="30" t="n">
+      <c r="L40" s="31" t="n">
         <v>1216.29</v>
       </c>
       <c r="M40" s="1" t="n"/>
@@ -4136,42 +4384,42 @@
       <c r="W40" s="1" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="55" t="inlineStr"/>
-      <c r="B41" s="29" t="inlineStr">
+      <c r="A41" s="56" t="inlineStr"/>
+      <c r="B41" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="C41" s="56" t="inlineStr">
+      <c r="C41" s="57" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="D41" s="59" t="n">
+      <c r="D41" s="60" t="n">
         <v>122.12</v>
       </c>
-      <c r="E41" s="30" t="n">
+      <c r="E41" s="31" t="n">
         <v>818371.29</v>
       </c>
-      <c r="F41" s="30" t="n">
+      <c r="F41" s="31" t="n">
         <v>6701.28</v>
       </c>
-      <c r="G41" s="31" t="n">
+      <c r="G41" s="32" t="n">
         <v>0.0338</v>
       </c>
-      <c r="H41" s="30" t="n">
+      <c r="H41" s="31" t="n">
         <v>254316.41</v>
       </c>
-      <c r="I41" s="60" t="n">
+      <c r="I41" s="61" t="n">
         <v>0.3108</v>
       </c>
-      <c r="J41" s="30" t="n">
+      <c r="J41" s="31" t="n">
         <v>2082.49</v>
       </c>
-      <c r="K41" s="30" t="n">
+      <c r="K41" s="31" t="n">
         <v>14933</v>
       </c>
-      <c r="L41" s="30" t="n">
+      <c r="L41" s="31" t="n">
         <v>1040.56</v>
       </c>
       <c r="M41" s="1" t="n"/>
@@ -4187,42 +4435,42 @@
       <c r="W41" s="1" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="55" t="inlineStr"/>
-      <c r="B42" s="29" t="inlineStr">
+      <c r="A42" s="56" t="inlineStr"/>
+      <c r="B42" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C42" s="56" t="inlineStr">
+      <c r="C42" s="57" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="D42" s="59" t="n">
+      <c r="D42" s="60" t="n">
         <v>255.09</v>
       </c>
-      <c r="E42" s="30" t="n">
+      <c r="E42" s="31" t="n">
         <v>1844124.54</v>
       </c>
-      <c r="F42" s="30" t="n">
+      <c r="F42" s="31" t="n">
         <v>7229.4</v>
       </c>
-      <c r="G42" s="31" t="n">
+      <c r="G42" s="32" t="n">
         <v>0.0761</v>
       </c>
-      <c r="H42" s="30" t="n">
+      <c r="H42" s="31" t="n">
         <v>602778.74</v>
       </c>
-      <c r="I42" s="60" t="n">
+      <c r="I42" s="61" t="n">
         <v>0.3269</v>
       </c>
-      <c r="J42" s="30" t="n">
+      <c r="J42" s="31" t="n">
         <v>2363.04</v>
       </c>
-      <c r="K42" s="30" t="n">
+      <c r="K42" s="31" t="n">
         <v>25220</v>
       </c>
-      <c r="L42" s="30" t="n">
+      <c r="L42" s="31" t="n">
         <v>978.58</v>
       </c>
       <c r="M42" s="1" t="n"/>
@@ -4238,42 +4486,42 @@
       <c r="W42" s="1" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="55" t="inlineStr"/>
-      <c r="B43" s="29" t="inlineStr">
+      <c r="A43" s="56" t="inlineStr"/>
+      <c r="B43" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C43" s="56" t="inlineStr">
+      <c r="C43" s="57" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D43" s="59" t="n">
+      <c r="D43" s="60" t="n">
         <v>369.35</v>
       </c>
-      <c r="E43" s="30" t="n">
+      <c r="E43" s="31" t="n">
         <v>3048653.48</v>
       </c>
-      <c r="F43" s="30" t="n">
+      <c r="F43" s="31" t="n">
         <v>8254.049999999999</v>
       </c>
-      <c r="G43" s="31" t="n">
+      <c r="G43" s="32" t="n">
         <v>0.1258</v>
       </c>
-      <c r="H43" s="30" t="n">
+      <c r="H43" s="31" t="n">
         <v>985765.87</v>
       </c>
-      <c r="I43" s="60" t="n">
+      <c r="I43" s="61" t="n">
         <v>0.3233</v>
       </c>
-      <c r="J43" s="30" t="n">
+      <c r="J43" s="31" t="n">
         <v>2668.9</v>
       </c>
-      <c r="K43" s="30" t="n">
+      <c r="K43" s="31" t="n">
         <v>60800</v>
       </c>
-      <c r="L43" s="30" t="n">
+      <c r="L43" s="31" t="n">
         <v>1540.33</v>
       </c>
       <c r="M43" s="1" t="n"/>
@@ -4289,42 +4537,42 @@
       <c r="W43" s="1" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="55" t="inlineStr"/>
-      <c r="B44" s="29" t="inlineStr">
+      <c r="A44" s="56" t="inlineStr"/>
+      <c r="B44" s="30" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C44" s="56" t="inlineStr">
+      <c r="C44" s="57" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="D44" s="59" t="n">
+      <c r="D44" s="60" t="n">
         <v>241.48</v>
       </c>
-      <c r="E44" s="30" t="n">
+      <c r="E44" s="31" t="n">
         <v>1709754.85</v>
       </c>
-      <c r="F44" s="30" t="n">
+      <c r="F44" s="31" t="n">
         <v>7080.28</v>
       </c>
-      <c r="G44" s="31" t="n">
+      <c r="G44" s="32" t="n">
         <v>0.0706</v>
       </c>
-      <c r="H44" s="30" t="n">
+      <c r="H44" s="31" t="n">
         <v>560009.03</v>
       </c>
-      <c r="I44" s="60" t="n">
+      <c r="I44" s="61" t="n">
         <v>0.3275</v>
       </c>
-      <c r="J44" s="30" t="n">
+      <c r="J44" s="31" t="n">
         <v>2319.06</v>
       </c>
-      <c r="K44" s="30" t="n">
+      <c r="K44" s="31" t="n">
         <v>22083</v>
       </c>
-      <c r="L44" s="30" t="n">
+      <c r="L44" s="31" t="n">
         <v>919.03</v>
       </c>
       <c r="M44" s="1" t="n"/>
@@ -4340,42 +4588,42 @@
       <c r="W44" s="1" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="55" t="inlineStr"/>
-      <c r="B45" s="29" t="inlineStr">
+      <c r="A45" s="56" t="inlineStr"/>
+      <c r="B45" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C45" s="56" t="inlineStr">
+      <c r="C45" s="57" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D45" s="59" t="n">
+      <c r="D45" s="60" t="n">
         <v>260.41</v>
       </c>
-      <c r="E45" s="30" t="n">
+      <c r="E45" s="31" t="n">
         <v>1863775.69</v>
       </c>
-      <c r="F45" s="30" t="n">
+      <c r="F45" s="31" t="n">
         <v>7157.03</v>
       </c>
-      <c r="G45" s="31" t="n">
+      <c r="G45" s="32" t="n">
         <v>0.0769</v>
       </c>
-      <c r="H45" s="30" t="n">
+      <c r="H45" s="31" t="n">
         <v>625402.3</v>
       </c>
-      <c r="I45" s="60" t="n">
+      <c r="I45" s="61" t="n">
         <v>0.3356</v>
       </c>
-      <c r="J45" s="30" t="n">
+      <c r="J45" s="31" t="n">
         <v>2401.59</v>
       </c>
-      <c r="K45" s="30" t="n">
+      <c r="K45" s="31" t="n">
         <v>24923</v>
       </c>
-      <c r="L45" s="30" t="n">
+      <c r="L45" s="31" t="n">
         <v>889.59</v>
       </c>
       <c r="M45" s="1" t="n"/>
@@ -4391,42 +4639,42 @@
       <c r="W45" s="1" t="n"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="55" t="inlineStr"/>
-      <c r="B46" s="29" t="inlineStr">
+      <c r="A46" s="56" t="inlineStr"/>
+      <c r="B46" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C46" s="56" t="inlineStr">
+      <c r="C46" s="57" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D46" s="59" t="n">
+      <c r="D46" s="60" t="n">
         <v>338.5</v>
       </c>
-      <c r="E46" s="30" t="n">
+      <c r="E46" s="31" t="n">
         <v>2620797.34</v>
       </c>
-      <c r="F46" s="30" t="n">
+      <c r="F46" s="31" t="n">
         <v>7742.43</v>
       </c>
-      <c r="G46" s="31" t="n">
+      <c r="G46" s="32" t="n">
         <v>0.1082</v>
       </c>
-      <c r="H46" s="30" t="n">
+      <c r="H46" s="31" t="n">
         <v>876442.71</v>
       </c>
-      <c r="I46" s="60" t="n">
+      <c r="I46" s="61" t="n">
         <v>0.3344</v>
       </c>
-      <c r="J46" s="30" t="n">
+      <c r="J46" s="31" t="n">
         <v>2589.21</v>
       </c>
-      <c r="K46" s="30" t="n">
+      <c r="K46" s="31" t="n">
         <v>41783</v>
       </c>
-      <c r="L46" s="30" t="n">
+      <c r="L46" s="31" t="n">
         <v>1101.6</v>
       </c>
       <c r="M46" s="1" t="n"/>
@@ -4442,42 +4690,42 @@
       <c r="W46" s="1" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="55" t="inlineStr"/>
-      <c r="B47" s="29" t="inlineStr">
+      <c r="A47" s="56" t="inlineStr"/>
+      <c r="B47" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C47" s="56" t="inlineStr">
+      <c r="C47" s="57" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="D47" s="59" t="n">
+      <c r="D47" s="60" t="n">
         <v>307.34</v>
       </c>
-      <c r="E47" s="30" t="n">
+      <c r="E47" s="31" t="n">
         <v>2267018.63</v>
       </c>
-      <c r="F47" s="30" t="n">
+      <c r="F47" s="31" t="n">
         <v>7376.18</v>
       </c>
-      <c r="G47" s="31" t="n">
+      <c r="G47" s="32" t="n">
         <v>0.0936</v>
       </c>
-      <c r="H47" s="30" t="n">
+      <c r="H47" s="31" t="n">
         <v>763702.73</v>
       </c>
-      <c r="I47" s="60" t="n">
+      <c r="I47" s="61" t="n">
         <v>0.3369</v>
       </c>
-      <c r="J47" s="30" t="n">
+      <c r="J47" s="31" t="n">
         <v>2484.86</v>
       </c>
-      <c r="K47" s="30" t="n">
+      <c r="K47" s="31" t="n">
         <v>31533</v>
       </c>
-      <c r="L47" s="30" t="n">
+      <c r="L47" s="31" t="n">
         <v>963.58</v>
       </c>
       <c r="M47" s="1" t="n"/>
@@ -4493,42 +4741,42 @@
       <c r="W47" s="1" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="55" t="inlineStr"/>
-      <c r="B48" s="29" t="inlineStr">
+      <c r="A48" s="56" t="inlineStr"/>
+      <c r="B48" s="30" t="inlineStr">
         <is>
           <t>MBway</t>
         </is>
       </c>
-      <c r="C48" s="56" t="inlineStr">
+      <c r="C48" s="57" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D48" s="59" t="n">
+      <c r="D48" s="60" t="n">
         <v>398.78</v>
       </c>
-      <c r="E48" s="30" t="n">
+      <c r="E48" s="31" t="n">
         <v>3292150.8</v>
       </c>
-      <c r="F48" s="30" t="n">
+      <c r="F48" s="31" t="n">
         <v>8255.51</v>
       </c>
-      <c r="G48" s="31" t="n">
+      <c r="G48" s="32" t="n">
         <v>0.1359</v>
       </c>
-      <c r="H48" s="30" t="n">
+      <c r="H48" s="31" t="n">
         <v>1096393.82</v>
       </c>
-      <c r="I48" s="60" t="n">
+      <c r="I48" s="61" t="n">
         <v>0.333</v>
       </c>
-      <c r="J48" s="30" t="n">
+      <c r="J48" s="31" t="n">
         <v>2749.35</v>
       </c>
-      <c r="K48" s="30" t="n">
+      <c r="K48" s="31" t="n">
         <v>68291</v>
       </c>
-      <c r="L48" s="30" t="n">
+      <c r="L48" s="31" t="n">
         <v>1475.02</v>
       </c>
       <c r="M48" s="1" t="n"/>
@@ -4544,42 +4792,42 @@
       <c r="W48" s="1" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="55" t="inlineStr"/>
-      <c r="B49" s="29" t="inlineStr">
+      <c r="A49" s="56" t="inlineStr"/>
+      <c r="B49" s="30" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C49" s="56" t="inlineStr">
+      <c r="C49" s="57" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D49" s="59" t="n">
+      <c r="D49" s="60" t="n">
         <v>184.72</v>
       </c>
-      <c r="E49" s="30" t="n">
+      <c r="E49" s="31" t="n">
         <v>1191512.54</v>
       </c>
-      <c r="F49" s="30" t="n">
+      <c r="F49" s="31" t="n">
         <v>6450.49</v>
       </c>
-      <c r="G49" s="31" t="n">
+      <c r="G49" s="32" t="n">
         <v>0.0492</v>
       </c>
-      <c r="H49" s="30" t="n">
+      <c r="H49" s="31" t="n">
         <v>455099.2</v>
       </c>
-      <c r="I49" s="60" t="n">
+      <c r="I49" s="61" t="n">
         <v>0.382</v>
       </c>
-      <c r="J49" s="30" t="n">
+      <c r="J49" s="31" t="n">
         <v>2463.77</v>
       </c>
-      <c r="K49" s="30" t="n">
+      <c r="K49" s="31" t="n">
         <v>21968</v>
       </c>
-      <c r="L49" s="30" t="n">
+      <c r="L49" s="31" t="n">
         <v>1368.09</v>
       </c>
       <c r="M49" s="1" t="n"/>
@@ -4595,42 +4843,42 @@
       <c r="W49" s="1" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="55" t="inlineStr"/>
-      <c r="B50" s="29" t="inlineStr">
+      <c r="A50" s="56" t="inlineStr"/>
+      <c r="B50" s="30" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="C50" s="56" t="inlineStr">
+      <c r="C50" s="57" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D50" s="59" t="n">
+      <c r="D50" s="60" t="n">
         <v>236.95</v>
       </c>
-      <c r="E50" s="30" t="n">
+      <c r="E50" s="31" t="n">
         <v>1653869.91</v>
       </c>
-      <c r="F50" s="30" t="n">
+      <c r="F50" s="31" t="n">
         <v>6979.9</v>
       </c>
-      <c r="G50" s="31" t="n">
+      <c r="G50" s="32" t="n">
         <v>0.0683</v>
       </c>
-      <c r="H50" s="30" t="n">
+      <c r="H50" s="31" t="n">
         <v>626670.52</v>
       </c>
-      <c r="I50" s="60" t="n">
+      <c r="I50" s="61" t="n">
         <v>0.3789</v>
       </c>
-      <c r="J50" s="30" t="n">
+      <c r="J50" s="31" t="n">
         <v>2644.77</v>
       </c>
-      <c r="K50" s="30" t="n">
+      <c r="K50" s="31" t="n">
         <v>36612</v>
       </c>
-      <c r="L50" s="30" t="n">
+      <c r="L50" s="31" t="n">
         <v>1704.98</v>
       </c>
       <c r="M50" s="1" t="n"/>
@@ -4646,42 +4894,42 @@
       <c r="W50" s="1" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="55" t="inlineStr"/>
-      <c r="B51" s="29" t="inlineStr">
+      <c r="A51" s="56" t="inlineStr"/>
+      <c r="B51" s="30" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C51" s="56" t="inlineStr">
+      <c r="C51" s="57" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D51" s="59" t="n">
+      <c r="D51" s="60" t="n">
         <v>121.86</v>
       </c>
-      <c r="E51" s="30" t="n">
+      <c r="E51" s="31" t="n">
         <v>902399.37</v>
       </c>
-      <c r="F51" s="30" t="n">
+      <c r="F51" s="31" t="n">
         <v>7405.22</v>
       </c>
-      <c r="G51" s="31" t="n">
+      <c r="G51" s="32" t="n">
         <v>0.0372</v>
       </c>
-      <c r="H51" s="30" t="n">
+      <c r="H51" s="31" t="n">
         <v>178759.19</v>
       </c>
-      <c r="I51" s="60" t="n">
+      <c r="I51" s="61" t="n">
         <v>0.1981</v>
       </c>
-      <c r="J51" s="30" t="n">
+      <c r="J51" s="31" t="n">
         <v>1466.92</v>
       </c>
-      <c r="K51" s="30" t="n">
+      <c r="K51" s="31" t="n">
         <v>18850</v>
       </c>
-      <c r="L51" s="30" t="n">
+      <c r="L51" s="31" t="n">
         <v>1624.68</v>
       </c>
       <c r="M51" s="1" t="n"/>
@@ -4697,42 +4945,42 @@
       <c r="W51" s="1" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="55" t="inlineStr"/>
-      <c r="B52" s="29" t="inlineStr">
+      <c r="A52" s="56" t="inlineStr"/>
+      <c r="B52" s="30" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="C52" s="56" t="inlineStr">
+      <c r="C52" s="57" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D52" s="59" t="n">
+      <c r="D52" s="60" t="n">
         <v>143.56</v>
       </c>
-      <c r="E52" s="30" t="n">
+      <c r="E52" s="31" t="n">
         <v>1133628.58</v>
       </c>
-      <c r="F52" s="30" t="n">
+      <c r="F52" s="31" t="n">
         <v>7896.53</v>
       </c>
-      <c r="G52" s="31" t="n">
+      <c r="G52" s="32" t="n">
         <v>0.0468</v>
       </c>
-      <c r="H52" s="30" t="n">
+      <c r="H52" s="31" t="n">
         <v>220510.28</v>
       </c>
-      <c r="I52" s="60" t="n">
+      <c r="I52" s="61" t="n">
         <v>0.1945</v>
       </c>
-      <c r="J52" s="30" t="n">
+      <c r="J52" s="31" t="n">
         <v>1536.01</v>
       </c>
-      <c r="K52" s="30" t="n">
+      <c r="K52" s="31" t="n">
         <v>30240</v>
       </c>
-      <c r="L52" s="30" t="n">
+      <c r="L52" s="31" t="n">
         <v>2192.89</v>
       </c>
       <c r="M52" s="1" t="n"/>
@@ -4748,38 +4996,38 @@
       <c r="W52" s="1" t="n"/>
     </row>
     <row r="53" ht="17" customHeight="1">
-      <c r="A53" s="61" t="n"/>
-      <c r="B53" s="62" t="inlineStr">
+      <c r="A53" s="62" t="n"/>
+      <c r="B53" s="63" t="inlineStr">
         <is>
           <t>Total campus</t>
         </is>
       </c>
-      <c r="C53" s="61" t="n"/>
-      <c r="D53" s="63" t="n">
+      <c r="C53" s="62" t="n"/>
+      <c r="D53" s="64" t="n">
         <v>3253.62</v>
       </c>
-      <c r="E53" s="64" t="n">
+      <c r="E53" s="65" t="n">
         <v>24231703.55</v>
       </c>
-      <c r="F53" s="64" t="n">
+      <c r="F53" s="65" t="n">
         <v>7447.62</v>
       </c>
-      <c r="G53" s="65" t="n">
+      <c r="G53" s="66" t="n">
         <v>1</v>
       </c>
-      <c r="H53" s="64" t="n">
+      <c r="H53" s="65" t="n">
         <v>7831343.62</v>
       </c>
-      <c r="I53" s="66" t="n">
+      <c r="I53" s="67" t="n">
         <v>0.3232</v>
       </c>
-      <c r="J53" s="64" t="n">
+      <c r="J53" s="65" t="n">
         <v>2406.97</v>
       </c>
-      <c r="K53" s="64" t="n">
+      <c r="K53" s="65" t="n">
         <v>434174</v>
       </c>
-      <c r="L53" s="61" t="n"/>
+      <c r="L53" s="62" t="n"/>
       <c r="M53" s="1" t="n"/>
       <c r="N53" s="1" t="n"/>
       <c r="O53" s="1" t="n"/>
@@ -4793,24 +5041,24 @@
       <c r="W53" s="1" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="67" t="n"/>
-      <c r="B54" s="68" t="inlineStr">
+      <c r="A54" s="68" t="n"/>
+      <c r="B54" s="69" t="inlineStr">
         <is>
           <t>Siège et holding</t>
         </is>
       </c>
-      <c r="C54" s="67" t="n"/>
-      <c r="D54" s="67" t="n"/>
-      <c r="E54" s="67" t="n"/>
-      <c r="F54" s="67" t="n"/>
-      <c r="G54" s="67" t="n"/>
-      <c r="H54" s="69" t="n">
+      <c r="C54" s="68" t="n"/>
+      <c r="D54" s="68" t="n"/>
+      <c r="E54" s="68" t="n"/>
+      <c r="F54" s="68" t="n"/>
+      <c r="G54" s="68" t="n"/>
+      <c r="H54" s="70" t="n">
         <v>-3719839.98</v>
       </c>
-      <c r="I54" s="67" t="n"/>
-      <c r="J54" s="67" t="n"/>
-      <c r="K54" s="67" t="n"/>
-      <c r="L54" s="67" t="n"/>
+      <c r="I54" s="68" t="n"/>
+      <c r="J54" s="68" t="n"/>
+      <c r="K54" s="68" t="n"/>
+      <c r="L54" s="68" t="n"/>
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="n"/>
       <c r="O54" s="1" t="n"/>
@@ -4824,38 +5072,38 @@
       <c r="W54" s="1" t="n"/>
     </row>
     <row r="55" ht="19" customHeight="1">
-      <c r="A55" s="70" t="n"/>
-      <c r="B55" s="71" t="inlineStr">
+      <c r="A55" s="71" t="n"/>
+      <c r="B55" s="72" t="inlineStr">
         <is>
           <t>Groupe</t>
         </is>
       </c>
-      <c r="C55" s="70" t="n"/>
-      <c r="D55" s="72" t="n">
+      <c r="C55" s="71" t="n"/>
+      <c r="D55" s="73" t="n">
         <v>3253.62</v>
       </c>
-      <c r="E55" s="73" t="n">
+      <c r="E55" s="74" t="n">
         <v>24231703.55</v>
       </c>
-      <c r="F55" s="73" t="n">
+      <c r="F55" s="74" t="n">
         <v>7447.62</v>
       </c>
-      <c r="G55" s="74" t="n">
+      <c r="G55" s="75" t="n">
         <v>1</v>
       </c>
-      <c r="H55" s="73" t="n">
+      <c r="H55" s="74" t="n">
         <v>4111503.64</v>
       </c>
-      <c r="I55" s="75" t="n">
+      <c r="I55" s="76" t="n">
         <v>0.1697</v>
       </c>
-      <c r="J55" s="73" t="n">
+      <c r="J55" s="74" t="n">
         <v>1263.67</v>
       </c>
-      <c r="K55" s="73" t="n">
+      <c r="K55" s="74" t="n">
         <v>434174</v>
       </c>
-      <c r="L55" s="70" t="n"/>
+      <c r="L55" s="71" t="n"/>
       <c r="M55" s="1" t="n"/>
       <c r="N55" s="1" t="n"/>
       <c r="O55" s="1" t="n"/>
@@ -4895,7 +5143,7 @@
     </row>
     <row r="57" ht="12" customHeight="1">
       <c r="A57" s="1" t="n"/>
-      <c r="B57" s="48" t="inlineStr">
+      <c r="B57" s="49" t="inlineStr">
         <is>
           <t>Source : Tagetik TGK_MSSQL_07, scénario 2027BUD_V1.</t>
         </is>

</xml_diff>